<commit_message>
feat: integrate dual-source CP loader with Google Apps Script, early SN pre-check, and fix multi-qty modal SN fill loop
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/cp_data.xlsx
+++ b/projects/auto_page/autopageMKII/tables/cp_data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$N$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$P$32</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:P32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -508,6 +508,16 @@
           <t>last_updated</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>last_adjustment_method</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>suggested_cp</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -910,8 +920,236 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MNL-002435</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2737</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2609251AWCE1CK</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>CP2609160013 DC2608280030</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>2737</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:59:46</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>OC</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SP1-001567+SP1-001568+SP1-001569+SP1-001570</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>9036</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SP2-001858+SP2-001859</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1820</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SP2-001778+SP2-001779</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>832</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>CP2609040007 DC2609170010</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>9673</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SP4-000302</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>141</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>DC2609220006</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SP1-001445+SP1-001446+SP1-001447+SP1-001448</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>11997</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SP2-001869+SP2-001870</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>903</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SP2-001799+SP2-001800+SP2-001801+SP2-001802</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1849</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SP2-001749+SP2-001615+SP2-001616+SP2-001617</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1241</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SP2-001610+SP2-001611+SP2-001612+SP2-001613</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SP2-001858+SP2-001859</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1861</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>DC2608310029 DC2609140003</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SP2-001753+SP2-001755</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1449</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>955</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N16"/>
+  <autoFilter ref="A1:P32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: update date for test
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/cp_data.xlsx
+++ b/projects/auto_page/autopageMKII/tables/cp_data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$P$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$S$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P32"/>
+  <dimension ref="A1:S33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -518,6 +518,21 @@
           <t>suggested_cp</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>suggested_usage_start_date</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>suggested_usage_end_date</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>suggested_remark</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1001,155 +1016,200 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
+          <t>SP4-000302</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>9673</v>
+        <v>141</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>DC2609220006</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SP4-000302</t>
+          <t>SP2-001869+SP2-001870</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>141</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>23/09/2026</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>DC2609220006</t>
-        </is>
+        <v>903</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SP1-001445+SP1-001446+SP1-001447+SP1-001448</t>
+          <t>SP2-001799+SP2-001800+SP2-001801+SP2-001802</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>11997</v>
+        <v>1849</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SP2-001869+SP2-001870</t>
+          <t>SP2-001749+SP2-001615+SP2-001616+SP2-001617</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>903</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SP2-001799+SP2-001800+SP2-001801+SP2-001802</t>
+          <t>SP2-001858+SP2-001859</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1849</v>
+        <v>1861</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>DC2608310029 DC2609140003</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SP2-001749+SP2-001615+SP2-001616+SP2-001617</t>
+          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1241</v>
+        <v>950</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SP2-001610+SP2-001611+SP2-001612+SP2-001613</t>
+          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1234</v>
+        <v>955</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SP2-001858+SP2-001859</t>
+          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1861</v>
+        <v>9673</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>DC2608310029 DC2609140003</t>
+          <t>CP2609090005</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SP2-001753+SP2-001755</t>
+          <t>SP1-001445+SP1-001446+SP1-001447+SP1-001448</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1017</v>
+        <v>11997</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
+          <t>SP2-001753+SP2-001755</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>950</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
+          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1449</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+          <t>SP2-001610+SP2-001611+SP2-001612+SP2-001613</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>955</v>
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1449</v>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>CP2609220007</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>หมายเหตุ : Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1449</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P32"/>
+  <autoFilter ref="A1:S33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(accel & pricing): reorder Completed_Orders timestamp to col 1, enhance GAS CP sync & last_updated
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/cp_data.xlsx
+++ b/projects/auto_page/autopageMKII/tables/cp_data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$S$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$S$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S33"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -923,15 +923,20 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2609166YD777JH</t>
+          <t>260929A9FF4P5G</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-16 14:33:32</t>
+          <t>2026-10-01 11:11:03</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>OC</t>
         </is>
       </c>
     </row>
@@ -991,181 +996,296 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SP2-001778+SP2-001779</t>
+          <t>SP4-000302</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>832</v>
+        <v>141</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>CP2609040007 DC2609170010</t>
+          <t>DC2609220006</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SP4-000302</t>
+          <t>SP2-001869+SP2-001870</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>141</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>23/09/2026</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>DC2609220006</t>
-        </is>
+        <v>903</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SP2-001869+SP2-001870</t>
+          <t>SP2-001799+SP2-001800+SP2-001801+SP2-001802</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>903</v>
+        <v>1849</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SP2-001799+SP2-001800+SP2-001801+SP2-001802</t>
+          <t>SP2-001749+SP2-001615+SP2-001616+SP2-001617</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1849</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SP2-001749+SP2-001615+SP2-001616+SP2-001617</t>
+          <t>SP2-001858+SP2-001859</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1241</v>
+        <v>1861</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>DC2608310029 DC2609140003</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SP2-001858+SP2-001859</t>
+          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1861</v>
+        <v>9673</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>DC2608310029 DC2609140003</t>
+          <t>CP2609090005</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
+          <t>SP2-001778+SP2-001779</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>950</v>
+        <v>832</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>DC2609220002</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>23/09/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>09/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 832</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+          <t>SP2-001607+SP2-001754</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>955</v>
+        <v>794</v>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>DC2609220002</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>23/09/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>09/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 794</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
+          <t>PR5-000661</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>9673</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>08/10/2026</t>
-        </is>
+        <v>8602</v>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>CP2609090005</t>
+          <t>CP2609220002</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคา 8602</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SP1-001445+SP1-001446+SP1-001447+SP1-001448</t>
+          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>11997</v>
+        <v>9551</v>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>CP2609220002</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>23/09/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>09/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 9551</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SP2-001753+SP2-001755</t>
+          <t>SP1-001445+SP1-001446+SP1-001447+SP1-001448</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1017</v>
+        <v>11997</v>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>CP2609220007</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>23/09/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>09/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 11997</t>
+        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
+          <t>SP2-001803+SP2-001804+SP2-001805+SP2-001806</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1199</v>
+        <v>2931</v>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>CP2609220002</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>23/09/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>09/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 2931</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -1177,39 +1297,299 @@
       <c r="B32" t="n">
         <v>1234</v>
       </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>CP2609220007</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>23/09/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>09/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1234</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>950</v>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>CP2609220002</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>23/09/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>09/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 950</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1199</v>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>DC2609220006</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>23/09/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>09/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1199</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
         </is>
       </c>
-      <c r="B33" t="n">
+      <c r="B35" t="n">
         <v>1449</v>
       </c>
-      <c r="P33" t="inlineStr">
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>2026-10-01 11:50:55</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
         <is>
           <t>CP2609220007</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>23/09/2026</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>หมายเหตุ : Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1449</t>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>23/09/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>09/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1449</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SP2-001753+SP2-001755</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1017</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>2026-10-01 11:51:48</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>CP2609220007</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>23/09/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>09/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1017</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>955</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>2026-10-01 11:53:19</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>CP2609220002</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>23/09/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>09/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 955</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1477</v>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>2026-10-01 11:57:20</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>01/10/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>31/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1477</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>969</v>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>2026-10-01 11:58:29</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>01/10/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>31/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 969</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>974</v>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>2026-10-01 11:59:34</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>01/10/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>31/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 974</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S33"/>
+  <autoFilter ref="A1:S40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: make jev skill be used serriopusly
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/cp_data.xlsx
+++ b/projects/auto_page/autopageMKII/tables/cp_data.xlsx
@@ -1381,15 +1381,15 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
+          <t>SP2-001753+SP2-001755</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1449</v>
+        <v>1017</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-10-01 11:50:55</t>
+          <t>2026-10-01 11:51:48</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -1409,27 +1409,27 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1449</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1017</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SP2-001753+SP2-001755</t>
+          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1017</v>
+        <v>955</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-10-01 11:51:48</t>
+          <t>2026-10-01 11:53:19</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -1444,62 +1444,62 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1017</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 955</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>955</v>
+        <v>1477</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-10-01 11:53:19</t>
+          <t>2026-10-01 11:57:20</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>23/09/2026 00:00:01</t>
+          <t>01/10/2026 00:00:01</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>09/10/2026 23:59:59</t>
+          <t>31/10/2026 23:59:59</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 955</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1477</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
+          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1477</v>
+        <v>969</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-10-01 11:57:20</t>
+          <t>2026-10-01 11:58:29</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
+          <t>CP2609290081</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -1514,22 +1514,22 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1477</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 969</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
+          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>969</v>
+        <v>974</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-10-01 11:58:29</t>
+          <t>2026-10-01 11:59:34</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -1549,42 +1549,42 @@
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 969</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 974</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>974</v>
+        <v>1449</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-10-01 11:59:34</t>
+          <t>2026-10-01 17:06:31</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>01/10/2026 00:00:01</t>
+          <t>23/09/2026 00:00:01</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>31/10/2026 23:59:59</t>
+          <t>09/10/2026 23:59:59</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 974</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1449</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(cp_data): remove redundant individual sub-SKU rows and consolidate into combo row
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/cp_data.xlsx
+++ b/projects/auto_page/autopageMKII/tables/cp_data.xlsx
@@ -9,17 +9,16 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$S$44</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -59,13 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,11 +429,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S44"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -548,12 +543,26 @@
           <t xml:space="preserve">DC2608210007 </t>
         </is>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="2" t="n">
         <v>46258</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="2" t="n">
         <v>46273</v>
       </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -569,12 +578,26 @@
           <t xml:space="preserve">DC2607310017 </t>
         </is>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="2" t="n">
         <v>46235</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="2" t="n">
         <v>46273</v>
       </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -585,6 +608,14 @@
       <c r="B4" t="n">
         <v>143</v>
       </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>2609141SRMKUEH</t>
@@ -603,6 +634,11 @@
           <t>2026-09-14 14:53:23</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -613,6 +649,14 @@
       <c r="B5" t="n">
         <v>300</v>
       </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>2609141MCF7RSD</t>
@@ -631,6 +675,11 @@
           <t>2026-09-14 14:48:42</t>
         </is>
       </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -641,6 +690,14 @@
       <c r="B6" t="n">
         <v>300</v>
       </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>2609141MCF7RSD</t>
@@ -659,6 +716,11 @@
           <t>2026-09-14 14:48:42</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -669,6 +731,14 @@
       <c r="B7" t="n">
         <v>301</v>
       </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>2609141MCF7RSD</t>
@@ -687,6 +757,11 @@
           <t>2026-09-14 14:48:42</t>
         </is>
       </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -697,6 +772,14 @@
       <c r="B8" t="n">
         <v>301</v>
       </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>2609141MCF7RSD</t>
@@ -715,6 +798,11 @@
           <t>2026-09-14 14:48:42</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -725,6 +813,14 @@
       <c r="B9" t="n">
         <v>1404</v>
       </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>2609141P1CYP3G</t>
@@ -743,6 +839,11 @@
           <t>2026-09-14 14:51:36</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -753,6 +854,14 @@
       <c r="B10" t="n">
         <v>311</v>
       </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>2609141P4RQJXW</t>
@@ -771,6 +880,11 @@
           <t>2026-09-14 14:57:10</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -781,6 +895,14 @@
       <c r="B11" t="n">
         <v>310</v>
       </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>2609141P4RQJXW</t>
@@ -799,6 +921,11 @@
           <t>2026-09-14 14:57:10</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -809,6 +936,14 @@
       <c r="B12" t="n">
         <v>310</v>
       </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>2609141P4RQJXW</t>
@@ -827,6 +962,11 @@
           <t>2026-09-14 14:57:10</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -837,6 +977,14 @@
       <c r="B13" t="n">
         <v>311</v>
       </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>2609141P4RQJXW</t>
@@ -855,6 +1003,11 @@
           <t>2026-09-14 14:57:10</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -865,6 +1018,14 @@
       <c r="B14" t="n">
         <v>390</v>
       </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>2609141KA8DDEA</t>
@@ -883,6 +1044,11 @@
           <t>2026-09-14 15:05:24</t>
         </is>
       </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -893,6 +1059,14 @@
       <c r="B15" t="n">
         <v>594</v>
       </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>2609141KA8DDEA</t>
@@ -911,6 +1085,11 @@
           <t>2026-09-14 15:05:24</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -921,11 +1100,20 @@
       <c r="B16" t="n">
         <v>4</v>
       </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>260929A9FF4P5G</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
         <v>4</v>
       </c>
@@ -939,6 +1127,10 @@
           <t>OC</t>
         </is>
       </c>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -949,6 +1141,14 @@
       <c r="B17" t="n">
         <v>2737</v>
       </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>2609251AWCE1CK</t>
@@ -972,6 +1172,10 @@
           <t>OC</t>
         </is>
       </c>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -982,6 +1186,23 @@
       <c r="B18" t="n">
         <v>9036</v>
       </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -992,6 +1213,23 @@
       <c r="B19" t="n">
         <v>1820</v>
       </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1002,6 +1240,7 @@
       <c r="B20" t="n">
         <v>141</v>
       </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>23/09/2026</t>
@@ -1012,11 +1251,24 @@
           <t>09/10/2026</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
           <t>DC2609220006</t>
         </is>
       </c>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1027,6 +1279,23 @@
       <c r="B21" t="n">
         <v>903</v>
       </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1037,6 +1306,23 @@
       <c r="B22" t="n">
         <v>1849</v>
       </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1047,6 +1333,23 @@
       <c r="B23" t="n">
         <v>1241</v>
       </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1057,6 +1360,7 @@
       <c r="B24" t="n">
         <v>1861</v>
       </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>14/09/2026</t>
@@ -1067,11 +1371,24 @@
           <t>30/09/2026</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
           <t>DC2608310029 DC2609140003</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1082,6 +1399,7 @@
       <c r="B25" t="n">
         <v>9673</v>
       </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>09/09/2026</t>
@@ -1092,11 +1410,24 @@
           <t>08/10/2026</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
           <t>CP2609090005</t>
         </is>
       </c>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1107,6 +1438,7 @@
       <c r="B26" t="n">
         <v>832</v>
       </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>18/09/2026</t>
@@ -1117,6 +1449,16 @@
           <t>08/10/2026</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
           <t>DC2609220002</t>
@@ -1147,6 +1489,19 @@
       <c r="B27" t="n">
         <v>794</v>
       </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
           <t>DC2609220002</t>
@@ -1177,6 +1532,19 @@
       <c r="B28" t="n">
         <v>8602</v>
       </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
           <t>CP2609220002</t>
@@ -1207,6 +1575,19 @@
       <c r="B29" t="n">
         <v>9551</v>
       </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
           <t>CP2609220002</t>
@@ -1237,6 +1618,19 @@
       <c r="B30" t="n">
         <v>11997</v>
       </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
           <t>CP2609220007</t>
@@ -1267,6 +1661,19 @@
       <c r="B31" t="n">
         <v>2931</v>
       </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
           <t>CP2609220002</t>
@@ -1297,6 +1704,19 @@
       <c r="B32" t="n">
         <v>1234</v>
       </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
           <t>CP2609220007</t>
@@ -1327,6 +1747,19 @@
       <c r="B33" t="n">
         <v>950</v>
       </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
           <t>CP2609220002</t>
@@ -1357,6 +1790,19 @@
       <c r="B34" t="n">
         <v>1199</v>
       </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
           <t>DC2609220006</t>
@@ -1387,11 +1833,23 @@
       <c r="B35" t="n">
         <v>1017</v>
       </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
           <t>2026-10-01 11:51:48</t>
         </is>
       </c>
+      <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
           <t>CP2609220007</t>
@@ -1422,11 +1880,23 @@
       <c r="B36" t="n">
         <v>955</v>
       </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
           <t>2026-10-01 11:53:19</t>
         </is>
       </c>
+      <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
           <t>CP2609220002</t>
@@ -1457,11 +1927,23 @@
       <c r="B37" t="n">
         <v>1477</v>
       </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
           <t>2026-10-01 11:57:20</t>
         </is>
       </c>
+      <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
           <t>CP2609300040</t>
@@ -1492,11 +1974,23 @@
       <c r="B38" t="n">
         <v>969</v>
       </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
           <t>2026-10-01 11:58:29</t>
         </is>
       </c>
+      <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
         <is>
           <t>CP2609290081</t>
@@ -1527,11 +2021,23 @@
       <c r="B39" t="n">
         <v>974</v>
       </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr">
         <is>
           <t>2026-10-01 11:59:34</t>
         </is>
       </c>
+      <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
           <t>CP2609290081</t>
@@ -1562,11 +2068,23 @@
       <c r="B40" t="n">
         <v>1449</v>
       </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
         <is>
           <t>2026-10-01 17:06:31</t>
         </is>
       </c>
+      <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
         <is>
           <t>CP2609220007</t>
@@ -1588,140 +2106,7 @@
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>SP2-001792</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>363</v>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>2609287HFYKV3U</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>CP2609220007</t>
-        </is>
-      </c>
-      <c r="M41" t="n">
-        <v>363</v>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>2026-10-01 17:58:23</t>
-        </is>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>CP</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>SP2-001793</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>362</v>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>2609287HFYKV3U</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>CP2609220007</t>
-        </is>
-      </c>
-      <c r="M42" t="n">
-        <v>362</v>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>2026-10-01 17:58:23</t>
-        </is>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>CP</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>SP2-001794</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>362</v>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>2609287HFYKV3U</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>CP2609220007</t>
-        </is>
-      </c>
-      <c r="M43" t="n">
-        <v>362</v>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>2026-10-01 17:58:23</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>CP</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>SP2-001795</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>362</v>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>2609287HFYKV3U</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>CP2609220007</t>
-        </is>
-      </c>
-      <c r="M44" t="n">
-        <v>362</v>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>2026-10-01 17:58:23</t>
-        </is>
-      </c>
-      <c r="O44" t="inlineStr">
-        <is>
-          <t>CP</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:S44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(pricing): record Auto-Learn CP data based on Order SKUs instead of raw POS cart items and skip shipping SKUs
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/cp_data.xlsx
+++ b/projects/auto_page/autopageMKII/tables/cp_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S40"/>
+  <dimension ref="A1:S39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1094,11 +1094,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SV0-000101</t>
+          <t>MNL-002435</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4</v>
+        <v>2737</v>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
@@ -1110,16 +1110,20 @@
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>260929A9FF4P5G</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr"/>
+          <t>2609251AWCE1CK</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>CP2609160013 DC2608280030</t>
+        </is>
+      </c>
       <c r="M16" t="n">
-        <v>4</v>
+        <v>2737</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-10-01 11:11:03</t>
+          <t>2026-09-29 14:59:46</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1135,11 +1139,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MNL-002435</t>
+          <t>SP1-001567+SP1-001568+SP1-001569+SP1-001570</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2737</v>
+        <v>9036</v>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
@@ -1149,29 +1153,11 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>2609251AWCE1CK</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>CP2609160013 DC2608280030</t>
-        </is>
-      </c>
-      <c r="M17" t="n">
-        <v>2737</v>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>2026-09-29 14:59:46</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>OC</t>
-        </is>
-      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
@@ -1180,11 +1166,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SP1-001567+SP1-001568+SP1-001569+SP1-001570</t>
+          <t>SP2-001858+SP2-001859</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>9036</v>
+        <v>1820</v>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
@@ -1207,15 +1193,23 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SP2-001858+SP2-001859</t>
+          <t>SP4-000302</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1820</v>
+        <v>141</v>
       </c>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
@@ -1226,7 +1220,11 @@
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>DC2609220006</t>
+        </is>
+      </c>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
@@ -1234,23 +1232,15 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SP4-000302</t>
+          <t>SP2-001869+SP2-001870</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>141</v>
+        <v>903</v>
       </c>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>23/09/2026</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
@@ -1261,11 +1251,7 @@
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>DC2609220006</t>
-        </is>
-      </c>
+      <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
@@ -1273,11 +1259,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SP2-001869+SP2-001870</t>
+          <t>SP2-001799+SP2-001800+SP2-001801+SP2-001802</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>903</v>
+        <v>1849</v>
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
@@ -1300,11 +1286,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SP2-001799+SP2-001800+SP2-001801+SP2-001802</t>
+          <t>SP2-001749+SP2-001615+SP2-001616+SP2-001617</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1849</v>
+        <v>1241</v>
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
@@ -1327,15 +1313,23 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SP2-001749+SP2-001615+SP2-001616+SP2-001617</t>
+          <t>SP2-001858+SP2-001859</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1241</v>
+        <v>1861</v>
       </c>
       <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -1346,7 +1340,11 @@
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>DC2608310029 DC2609140003</t>
+        </is>
+      </c>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
@@ -1354,21 +1352,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SP2-001858+SP2-001859</t>
+          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1861</v>
+        <v>9673</v>
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
@@ -1383,7 +1381,7 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
-          <t>DC2608310029 DC2609140003</t>
+          <t>CP2609090005</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr"/>
@@ -1393,16 +1391,16 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
+          <t>SP2-001778+SP2-001779</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>9673</v>
+        <v>832</v>
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1422,33 +1420,37 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
-          <t>CP2609090005</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
+          <t>DC2609220002</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>23/09/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>09/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 832</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SP2-001778+SP2-001779</t>
+          <t>SP2-001607+SP2-001754</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>832</v>
+        <v>794</v>
       </c>
       <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>18/09/2026</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>08/10/2026</t>
-        </is>
-      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
@@ -1476,18 +1478,18 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 832</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 794</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SP2-001607+SP2-001754</t>
+          <t>PR5-000661</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>794</v>
+        <v>8602</v>
       </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
@@ -1504,33 +1506,33 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
-          <t>DC2609220002</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>23/09/2026 00:00:01</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>09/10/2026 23:59:59</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 794</t>
+          <t>Shp/TT เดือน ก.ย. ราคา 8602</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PR5-000661</t>
+          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>8602</v>
+        <v>9551</v>
       </c>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
@@ -1552,28 +1554,28 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>23/09/2026 00:00:01</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>09/10/2026 23:59:59</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคา 8602</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 9551</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
+          <t>SP1-001445+SP1-001446+SP1-001447+SP1-001448</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>9551</v>
+        <v>11997</v>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
@@ -1590,7 +1592,7 @@
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -1605,18 +1607,18 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 9551</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 11997</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SP1-001445+SP1-001446+SP1-001447+SP1-001448</t>
+          <t>SP2-001803+SP2-001804+SP2-001805+SP2-001806</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>11997</v>
+        <v>2931</v>
       </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
@@ -1633,7 +1635,7 @@
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -1648,18 +1650,18 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 11997</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 2931</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SP2-001803+SP2-001804+SP2-001805+SP2-001806</t>
+          <t>SP2-001610+SP2-001611+SP2-001612+SP2-001613</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2931</v>
+        <v>1234</v>
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
@@ -1676,7 +1678,7 @@
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -1691,18 +1693,18 @@
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 2931</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1234</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SP2-001610+SP2-001611+SP2-001612+SP2-001613</t>
+          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1234</v>
+        <v>950</v>
       </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
@@ -1719,7 +1721,7 @@
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -1734,18 +1736,18 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1234</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 950</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
+          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>950</v>
+        <v>1199</v>
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
@@ -1762,7 +1764,7 @@
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
+          <t>DC2609220006</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -1777,18 +1779,18 @@
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 950</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1199</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
+          <t>SP2-001753+SP2-001755</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1199</v>
+        <v>1017</v>
       </c>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
@@ -1801,11 +1803,15 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>2026-10-01 11:51:48</t>
+        </is>
+      </c>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
-          <t>DC2609220006</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -1820,18 +1826,18 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1199</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1017</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SP2-001753+SP2-001755</t>
+          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1017</v>
+        <v>955</v>
       </c>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
@@ -1846,13 +1852,13 @@
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-10-01 11:51:48</t>
+          <t>2026-10-01 11:53:19</t>
         </is>
       </c>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -1867,18 +1873,18 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1017</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 955</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>955</v>
+        <v>1477</v>
       </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
@@ -1893,39 +1899,39 @@
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-10-01 11:53:19</t>
+          <t>2026-10-01 11:57:20</t>
         </is>
       </c>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>23/09/2026 00:00:01</t>
+          <t>01/10/2026 00:00:01</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>09/10/2026 23:59:59</t>
+          <t>31/10/2026 23:59:59</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 955</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1477</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
+          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1477</v>
+        <v>969</v>
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
@@ -1940,13 +1946,13 @@
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-10-01 11:57:20</t>
+          <t>2026-10-01 11:58:29</t>
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
+          <t>CP2609290081</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
@@ -1961,18 +1967,18 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1477</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 969</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
+          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>969</v>
+        <v>974</v>
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
@@ -1987,7 +1993,7 @@
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-10-01 11:58:29</t>
+          <t>2026-10-01 11:59:34</t>
         </is>
       </c>
       <c r="O38" t="inlineStr"/>
@@ -2008,18 +2014,18 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 969</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 974</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>974</v>
+        <v>1449</v>
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
@@ -2034,73 +2040,26 @@
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-10-01 11:59:34</t>
+          <t>2026-10-01 17:06:31</t>
         </is>
       </c>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>01/10/2026 00:00:01</t>
+          <t>23/09/2026 00:00:01</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>31/10/2026 23:59:59</t>
+          <t>09/10/2026 23:59:59</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 974</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>1449</v>
-      </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>2026-10-01 17:06:31</t>
-        </is>
-      </c>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>CP2609220007</t>
-        </is>
-      </c>
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t>23/09/2026 00:00:01</t>
-        </is>
-      </c>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>09/10/2026 23:59:59</t>
-        </is>
-      </c>
-      <c r="S40" t="inlineStr">
         <is>
           <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1449</t>
         </is>

</xml_diff>

<commit_message>
feat(pricing, payment, session): add realtime cp ambiguity detection, topmost mismatch dialog, and session timer on close
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/cp_data.xlsx
+++ b/projects/auto_page/autopageMKII/tables/cp_data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$S$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$S$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S56"/>
+  <dimension ref="A1:S57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>261001FGRN0E3U</t>
+          <t>261004QX1BTQAW</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-10-02 16:23:56</t>
+          <t>2026-10-05 15:15:04</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>261001G5NXM272</t>
+          <t>261005SPK3PU2U</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-10-02 17:51:08</t>
+          <t>2026-10-05 15:36:58</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>261002HSQNAN0G</t>
+          <t>261005S1000PVF</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-10-02 18:01:03</t>
+          <t>2026-10-05 16:09:48</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>261001GGR265EJ</t>
+          <t>261005S561P3G2</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-10-02 17:54:59</t>
+          <t>2026-10-05 15:23:04</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>261001EXVBHTNJ</t>
+          <t>261005SGFV6AYU</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026-10-02 16:20:06</t>
+          <t>2026-10-05 15:32:13</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
@@ -2230,7 +2230,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>261002HNMRU6N2</t>
+          <t>261005SRV913UJ</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026-10-02 17:59:34</t>
+          <t>2026-10-05 15:37:57</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
@@ -2395,9 +2395,27 @@
           <t>31/10/2026</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>261005SB6KAGSA</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="M48" t="n">
+        <v>3031</v>
+      </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>2026-10-02 16:21:12</t>
+          <t>2026-10-05 15:28:13</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -2447,7 +2465,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>261003ND0STEU0</t>
+          <t>261005SEX8B805</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -2460,7 +2478,7 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>2026-10-05 10:38:45</t>
+          <t>2026-10-05 15:30:39</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
@@ -2596,7 +2614,7 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>2026-10-05 10:37:22</t>
+          <t>2026-10-05 15:07:40</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
@@ -2684,7 +2702,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>261001FX5EERNK</t>
+          <t>261004PYNMBJ77</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -2697,7 +2715,7 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>2026-10-02 17:48:15</t>
+          <t>2026-10-05 15:09:51</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
@@ -2803,6 +2821,21 @@
       <c r="B55" t="n">
         <v>305</v>
       </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>DC2609300024</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
       <c r="N55" t="inlineStr">
         <is>
           <t>2026-10-02 17:42:36</t>
@@ -2832,20 +2865,138 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>SP2-001748+SP2-001615+SP2-001616+SP2-001617</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1330</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>DC2609290042</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>261005S1000PVF</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>DC2609290042</t>
+        </is>
+      </c>
+      <c r="M56" t="n">
+        <v>1330</v>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>2026-10-05 16:09:48</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>DC2609290042</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>01/10/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>31/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 1330</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>SP2-001753+SP2-001755</t>
         </is>
       </c>
-      <c r="B56" t="n">
+      <c r="B57" t="n">
         <v>993</v>
       </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>2026-10-05 10:37:56</t>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>CP2609140012</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46279.00001157408</v>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>5 4</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>261005SER9K7CC</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>CP2609140012</t>
+        </is>
+      </c>
+      <c r="M57" t="n">
+        <v>993</v>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>2026-10-05 16:34:34</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>CP + OC</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>CP2610050027</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>FS Shp Rebate ราคาเซ็ทละ 993</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S56"/>
+  <autoFilter ref="A1:S57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: ปรับ logic การupdate cp_data
suggested_remark ไม่มีการ update ตาม cp ใน smco มัโชว์ remark cp เดิมเสมอไม่อัพเดทเมื่อ cp_remark เปนอันใหม่
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/cp_data.xlsx
+++ b/projects/auto_page/autopageMKII/tables/cp_data.xlsx
@@ -1590,7 +1590,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>261005SPK3PU2U</t>
+          <t>261004R3TD9APG</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-10-05 15:36:58</t>
+          <t>2026-10-07 14:38:24</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -2207,79 +2207,44 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SP4-000302</t>
+          <t>MS2-000754</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>139</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>DC2609300024</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>31/10/2026</t>
-        </is>
+        <v>375</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>261005SRV913UJ</t>
+          <t>260929BD1UJHCV</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>DC2609300024</t>
+          <t>CP2609290069 DC2609290002</t>
         </is>
       </c>
       <c r="M44" t="n">
-        <v>139</v>
+        <v>375</v>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026-10-05 15:37:57</t>
+          <t>2026-10-02 16:35:35</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>CP</t>
-        </is>
-      </c>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>DC2609300024</t>
-        </is>
-      </c>
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>31/10/2026</t>
-        </is>
-      </c>
-      <c r="S44" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ต.ค. ราคา 139</t>
+          <t>OC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>MS2-000754</t>
+          <t>MS2-000820</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>375</v>
+        <v>225</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -2292,7 +2257,7 @@
         </is>
       </c>
       <c r="M45" t="n">
-        <v>375</v>
+        <v>225</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
@@ -2301,18 +2266,18 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>OC</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>MS2-000820</t>
+          <t>MS2-000942</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>225</v>
+        <v>450</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
@@ -2325,7 +2290,7 @@
         </is>
       </c>
       <c r="M46" t="n">
-        <v>225</v>
+        <v>450</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
@@ -2341,76 +2306,111 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MS2-000942</t>
+          <t>SP1-001378</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>450</v>
+        <v>3031</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>260929BD1UJHCV</t>
+          <t>261005SB6KAGSA</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>CP2609290069 DC2609290002</t>
+          <t>CP2609290081</t>
         </is>
       </c>
       <c r="M47" t="n">
-        <v>450</v>
+        <v>3031</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>2026-10-02 16:35:35</t>
+          <t>2026-10-05 15:28:13</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 3031</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SP1-001378</t>
+          <t>SP2-001610+SP2-001611+SP2-001612+SP2-001613</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>3031</v>
+        <v>1280</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>01/10/2026 00:00:01</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>31/10/2026</t>
+          <t>31/10/2026 23:59:59</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>261005SB6KAGSA</t>
+          <t>261005SEX8B805</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="M48" t="n">
-        <v>3031</v>
+        <v>1280</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>2026-10-05 15:28:13</t>
+          <t>2026-10-05 15:30:39</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
@@ -2420,65 +2420,65 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>01/10/2026 00:00:01</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>31/10/2026</t>
+          <t>31/10/2026 23:59:59</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคา 3031</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1280</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SP2-001610+SP2-001611+SP2-001612+SP2-001613</t>
+          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1280</v>
+        <v>9673</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
+          <t>CP2609090005</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>01/10/2026 00:00:01</t>
+          <t>09/09/2026 00:00:01</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>31/10/2026 23:59:59</t>
+          <t>08/10/2026 23:59:59</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>261005SEX8B805</t>
+          <t>261001FNX3QHKT</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
+          <t>CP2609090005</t>
         </is>
       </c>
       <c r="M49" t="n">
-        <v>1280</v>
+        <v>9673</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>2026-10-05 15:30:39</t>
+          <t>2026-10-02 17:47:09</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
@@ -2488,65 +2488,65 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
+          <t>CP2609090005</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>01/10/2026 00:00:01</t>
+          <t>09/09/2026 00:00:01</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>31/10/2026 23:59:59</t>
+          <t>08/10/2026 23:59:59</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1280</t>
+          <t>Dynamic ก.ย. Shp ราคา 9673</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
+          <t>SP2-001753+SP2-001755</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>9673</v>
+        <v>1056</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>CP2609090005</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>09/09/2026 00:00:01</t>
+          <t>01/10/2026 00:00:01</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>08/10/2026 23:59:59</t>
+          <t>31/10/2026 23:59:59</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>261001FNX3QHKT</t>
+          <t>261002JEPP9507</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>CP2609090005</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="M50" t="n">
-        <v>9673</v>
+        <v>1056</v>
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>2026-10-02 17:47:09</t>
+          <t>2026-10-07 14:36:59</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
@@ -2556,134 +2556,129 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>CP2609090005</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>09/09/2026 00:00:01</t>
+          <t>01/10/2026 00:00:01</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>08/10/2026 23:59:59</t>
-        </is>
-      </c>
-      <c r="S50" t="inlineStr">
-        <is>
-          <t>Dynamic ก.ย. Shp ราคา 9673</t>
+          <t>31/10/2026 23:59:59</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SP2-001753+SP2-001755</t>
+          <t>MNL-002445</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1056</v>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>CP2609300040</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>01/10/2026 00:00:01</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>31/10/2026 23:59:59</t>
-        </is>
+        <v>2847</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>261002JEPP9507</t>
+          <t>261001FVHQUH0S</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
+          <t>CP2609280021 DC2609280008</t>
         </is>
       </c>
       <c r="M51" t="n">
-        <v>1056</v>
+        <v>2847</v>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>2026-10-05 15:07:40</t>
+          <t>2026-10-02 16:32:59</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>CP</t>
-        </is>
-      </c>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t>CP2609300040</t>
-        </is>
-      </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>01/10/2026 00:00:01</t>
-        </is>
-      </c>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>31/10/2026 23:59:59</t>
-        </is>
-      </c>
-      <c r="S51" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ต.ค. ราคา 409</t>
+          <t>OC</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>MNL-002445</t>
+          <t>SP1-001210</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2847</v>
+        <v>1446</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>261001FVHQUH0S</t>
+          <t>261004PYNMBJ77</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>CP2609280021 DC2609280008</t>
+          <t>DC2609290041</t>
         </is>
       </c>
       <c r="M52" t="n">
-        <v>2847</v>
+        <v>1446</v>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>2026-10-02 16:32:59</t>
+          <t>2026-10-05 15:09:51</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>OC</t>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 1446</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SP1-001210</t>
+          <t>SP1-001113</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1446</v>
+        <v>1603</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -2702,7 +2697,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>261004PYNMBJ77</t>
+          <t>261002HSH1MCYP</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -2711,11 +2706,11 @@
         </is>
       </c>
       <c r="M53" t="n">
-        <v>1446</v>
+        <v>1603</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>2026-10-05 15:09:51</t>
+          <t>2026-10-02 18:00:21</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
@@ -2740,22 +2735,22 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคา 1446</t>
+          <t>Shp/TT เดือน ต.ค. ราคา 1603</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SP1-001113</t>
+          <t>SP4-000196</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1603</v>
+        <v>305</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>DC2609290041</t>
+          <t>DC2609300024</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2768,32 +2763,14 @@
           <t>31/10/2026</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>261002HSH1MCYP</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>DC2609290041</t>
-        </is>
-      </c>
-      <c r="M54" t="n">
-        <v>1603</v>
-      </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>2026-10-02 18:00:21</t>
-        </is>
-      </c>
-      <c r="O54" t="inlineStr">
-        <is>
-          <t>CP</t>
+          <t>2026-10-02 17:42:36</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>DC2609290041</t>
+          <t>DC2609300024</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -2808,180 +2785,198 @@
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคา 1603</t>
+          <t>Shp/TT เดือน ต.ค. ราคา 305</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SP4-000196</t>
+          <t>SP2-001748+SP2-001615+SP2-001616+SP2-001617</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>305</v>
+        <v>1330</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>DC2609300024</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>31/10/2026</t>
-        </is>
+          <t>DC2609290042</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>261005S1000PVF</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>DC2609290042</t>
+        </is>
+      </c>
+      <c r="M55" t="n">
+        <v>1330</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>2026-10-02 17:42:36</t>
+          <t>2026-10-05 16:09:48</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>DC2609300024</t>
+          <t>DC2609290042</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>01/10/2026 00:00:01</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>31/10/2026</t>
+          <t>31/10/2026 23:59:59</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคา 305</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 1330</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SP2-001748+SP2-001615+SP2-001616+SP2-001617</t>
+          <t>SP2-001753+SP2-001755</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1330</v>
+        <v>993</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>DC2609290042</t>
+          <t>CP2609140012</t>
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46296.00001157408</v>
+        <v>46279.00001157408</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>46326.99998842592</v>
+        <v>46304</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>5 4</t>
+        </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>261005S1000PVF</t>
+          <t>261003K6J8B8H5</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>DC2609290042</t>
+          <t>CP2609140012</t>
         </is>
       </c>
       <c r="M56" t="n">
-        <v>1330</v>
+        <v>993</v>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>2026-10-05 16:09:48</t>
+          <t>2026-10-07 14:37:38</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>CP</t>
+          <t>CP + OC</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>DC2609290042</t>
+          <t>CP2610050027</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>01/10/2026 00:00:01</t>
+          <t>05/10/2026</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>31/10/2026 23:59:59</t>
+          <t>31/10/2026</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 1330</t>
+          <t>FS Shp Rebate ราคาเซ็ทละ 993</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SP2-001753+SP2-001755</t>
+          <t>SP4-000302</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>993</v>
+        <v>139</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>CP2609140012</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="n">
-        <v>46279.00001157408</v>
-      </c>
-      <c r="E57" s="3" t="n">
-        <v>46304</v>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>5 4</t>
+          <t>DC2609300024</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>261005SER9K7CC</t>
+          <t>261005SRV913UJ</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>CP2609140012</t>
+          <t>DC2609300024</t>
         </is>
       </c>
       <c r="M57" t="n">
-        <v>993</v>
+        <v>139</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>2026-10-05 16:34:34</t>
+          <t>2026-10-07 14:39:21</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>CP + OC</t>
+          <t>CP</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>CP2610050027</t>
+          <t>DC2609300024</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>05/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -2991,7 +2986,7 @@
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>FS Shp Rebate ราคาเซ็ทละ 993</t>
+          <t>Shp/TT เดือน ต.ค. ราคา 139</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(pos): separate distinct CP recipe patterns into individual rows and prevent oc/dc leak
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/cp_data.xlsx
+++ b/projects/auto_page/autopageMKII/tables/cp_data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$S$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$S$74</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S59"/>
+  <dimension ref="A1:S74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -556,7 +556,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>261002JEPP9507</t>
+          <t>261007265U804D</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-10-08 10:37:00</t>
+          <t>2026-10-08 11:11:26</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2610071GF09EGA</t>
+          <t>2610071YKH3P16</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-10-08 10:50:44</t>
+          <t>2026-10-08 11:07:28</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46296</v>
+        <v>46032</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>46326</v>
@@ -744,7 +744,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-10-08 10:53:27</t>
+          <t>2026-10-08 11:09:55</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -791,7 +791,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2610071KFTTTYK</t>
+          <t>26100729P4PHTQ</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-10-08 10:55:47</t>
+          <t>2026-10-08 11:15:29</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -869,17 +869,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-10-08 10:54:58</t>
+          <t>2026-10-08 11:13:37</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
           <t>CP + OC</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>CP2610050027</t>
         </is>
       </c>
       <c r="Q7" s="3" t="n">
@@ -888,11 +883,6 @@
       <c r="R7" s="3" t="n">
         <v>46337.99998842592</v>
       </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>FS Shp ถูกชัวร์ ราคาเซ็ทละ 993</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -916,7 +906,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2610071HRU9UPY</t>
+          <t>2610071PP00HWD</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -929,7 +919,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-10-08 10:52:36</t>
+          <t>2026-10-08 11:00:07</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -976,7 +966,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>261006V0FBP040</t>
+          <t>2610072A0U120S</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -989,7 +979,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-10-08 10:33:43</t>
+          <t>2026-10-08 11:17:02</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1299,14 +1289,14 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46296</v>
+        <v>46032</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>46326</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>26100717549GJX</t>
+          <t>2610071MEQQ7CT</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1319,7 +1309,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-10-08 10:38:43</t>
+          <t>2026-10-08 10:58:32</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1333,7 +1323,7 @@
         </is>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>46296</v>
+        <v>46032</v>
       </c>
       <c r="R16" s="3" t="n">
         <v>46326</v>
@@ -1347,887 +1337,799 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SP4-000302</t>
+          <t>SP2-001803+SP2-001804+SP2-001805+SP2-001806</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>137</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DC2608210007 </t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>46258</v>
-      </c>
-      <c r="E17" s="3" t="n">
-        <v>46273</v>
+        <v>2993</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>2026-10-08 10:59:18</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="Q17" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="R17" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 2993</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SP4-000242</t>
+          <t>TEST-PATTERN-SKU</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>860</v>
+        <v>999</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">DC2607310017 </t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>46030</v>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>46243</v>
+          <t>CP_INSERTED</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>08/10/2026 11:09:23</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SP4-000302</t>
+          <t>TEST-PATTERN-SKU-2</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>143</v>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>2609141SRMKUEH</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>DC2609140005</t>
-        </is>
-      </c>
-      <c r="M19" t="n">
-        <v>141</v>
+        <v>999</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CP_NEW</t>
+        </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-14 14:53:23</t>
+          <t>08/10/2026 11:02:06</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SP2-001713</t>
+          <t>SP2-001869+SP2-001870</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>300</v>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>2609141MCF7RSD</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>DC2609140005</t>
-        </is>
-      </c>
-      <c r="M20" t="n">
-        <v>300</v>
+        <v>921</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-14 14:48:42</t>
+          <t>2026-10-08 11:04:54</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="Q20" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="R20" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 921</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SP2-001714</t>
+          <t>SP1-001449</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>300</v>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>2609141MCF7RSD</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>DC2609140005</t>
-        </is>
-      </c>
-      <c r="M21" t="n">
-        <v>300</v>
+        <v>2220</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>DC2610010003</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>46336</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-09-14 14:48:42</t>
+          <t>2026-10-08 11:05:23</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>DC2610010003</t>
+        </is>
+      </c>
+      <c r="Q21" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R21" s="3" t="n">
+        <v>46336</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Shp+Lzd+Tiktok ราคา 2220</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SP2-001715</t>
+          <t>TEST-PATTERN-SKU</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>301</v>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>2609141MCF7RSD</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>DC2609140005</t>
-        </is>
-      </c>
-      <c r="M22" t="n">
-        <v>301</v>
+        <v>888</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CP_NEW_PRICE</t>
+        </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-14 14:48:42</t>
+          <t>08/10/2026 11:06:56</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SP2-001716</t>
+          <t>SP2-001778+SP2-001779</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>301</v>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>2609141MCF7RSD</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>DC2609140005</t>
-        </is>
-      </c>
-      <c r="M23" t="n">
-        <v>301</v>
+        <v>851</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>46326.99998842592</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-09-14 14:48:42</t>
+          <t>2026-10-08 11:09:24</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="Q23" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="R23" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 851</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SP1-001579</t>
+          <t>SP2-001607+SP2-001754</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1404</v>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>2609141P1CYP3G</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>DC2609140008</t>
-        </is>
-      </c>
-      <c r="M24" t="n">
-        <v>1404</v>
+        <v>810</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>46326.99998842592</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-14 14:51:36</t>
+          <t>2026-10-08 11:10:32</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="Q24" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="R24" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 810</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SP2-001610</t>
+          <t>MS2-000818</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>311</v>
+        <v>225</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CP2609290069 DC2609290002</t>
+        </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2609141P4RQJXW</t>
+          <t>261007288HJTKT</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>CP2609140012</t>
+          <t>CP2609290069 DC2609290002</t>
         </is>
       </c>
       <c r="M25" t="n">
-        <v>311</v>
+        <v>225</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-09-14 14:57:10</t>
+          <t>2026-10-08 11:12:30</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SP2-001611</t>
+          <t>SP4-000302</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>310</v>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>2609141P4RQJXW</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>CP2609140012</t>
-        </is>
-      </c>
-      <c r="M26" t="n">
-        <v>310</v>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>2026-09-14 14:57:10</t>
-        </is>
+        <v>137</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>DC2608210007</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>46258</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>46273</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SP2-001612</t>
+          <t>SP4-000242</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>310</v>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>2609141P4RQJXW</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>CP2609140012</t>
-        </is>
-      </c>
-      <c r="M27" t="n">
-        <v>310</v>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>2026-09-14 14:57:10</t>
-        </is>
+        <v>860</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>DC2607310017</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>46235</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>46273</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SP2-001613</t>
+          <t>SP4-000302</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>311</v>
+        <v>143</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2609141P4RQJXW</t>
+          <t>2609141SRMKUEH</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>CP2609140012</t>
+          <t>DC2609140005</t>
         </is>
       </c>
       <c r="M28" t="n">
-        <v>311</v>
+        <v>141</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-14 14:57:10</t>
+          <t>2026-09-14 14:53:23</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SP2-001753</t>
+          <t>SP2-001713</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>390</v>
+        <v>300</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2609141KA8DDEA</t>
+          <t>2609141MCF7RSD</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>CP2609140012</t>
+          <t>DC2609140005</t>
         </is>
       </c>
       <c r="M29" t="n">
-        <v>390</v>
+        <v>300</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-14 15:05:24</t>
+          <t>2026-09-14 14:48:42</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SP2-001755</t>
+          <t>SP2-001714</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>594</v>
+        <v>300</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2609141KA8DDEA</t>
+          <t>2609141MCF7RSD</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>CP2609140012</t>
+          <t>DC2609140005</t>
         </is>
       </c>
       <c r="M30" t="n">
-        <v>594</v>
+        <v>300</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-14 15:05:24</t>
+          <t>2026-09-14 14:48:42</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MNL-002435</t>
+          <t>SP2-001715</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2737</v>
+        <v>301</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2609251AWCE1CK</t>
+          <t>2609141MCF7RSD</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>CP2609160013 DC2608280030</t>
+          <t>DC2609140005</t>
         </is>
       </c>
       <c r="M31" t="n">
-        <v>2737</v>
+        <v>301</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-29 14:59:46</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>OC</t>
+          <t>2026-09-14 14:48:42</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SP1-001567+SP1-001568+SP1-001569+SP1-001570</t>
+          <t>SP2-001716</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>9036</v>
+        <v>301</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>2609141MCF7RSD</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>DC2609140005</t>
+        </is>
+      </c>
+      <c r="M32" t="n">
+        <v>301</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>2026-09-14 14:48:42</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SP2-001858+SP2-001859</t>
+          <t>SP1-001579</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1820</v>
+        <v>1404</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>2609141P1CYP3G</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>DC2609140008</t>
+        </is>
+      </c>
+      <c r="M33" t="n">
+        <v>1404</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>2026-09-14 14:51:36</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SP4-000302</t>
+          <t>SP2-001610</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>141</v>
-      </c>
-      <c r="D34" s="3" t="n">
-        <v>46288</v>
-      </c>
-      <c r="E34" s="3" t="n">
-        <v>46304</v>
-      </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>DC2609220006</t>
+        <v>311</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>2609141P4RQJXW</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>CP2609140012</t>
+        </is>
+      </c>
+      <c r="M34" t="n">
+        <v>311</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>2026-09-14 14:57:10</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SP2-001869+SP2-001870</t>
+          <t>SP2-001611</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>903</v>
+        <v>310</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>2609141P4RQJXW</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>CP2609140012</t>
+        </is>
+      </c>
+      <c r="M35" t="n">
+        <v>310</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>2026-09-14 14:57:10</t>
+        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SP2-001749+SP2-001615+SP2-001616+SP2-001617</t>
+          <t>SP2-001612</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1241</v>
+        <v>310</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>2609141P4RQJXW</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>CP2609140012</t>
+        </is>
+      </c>
+      <c r="M36" t="n">
+        <v>310</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>2026-09-14 14:57:10</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SP2-001858+SP2-001859</t>
+          <t>SP2-001613</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1861</v>
-      </c>
-      <c r="D37" s="3" t="n">
-        <v>46279</v>
-      </c>
-      <c r="E37" s="3" t="n">
-        <v>46295</v>
-      </c>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>DC2608310029 DC2609140003</t>
+        <v>311</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>2609141P4RQJXW</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>CP2609140012</t>
+        </is>
+      </c>
+      <c r="M37" t="n">
+        <v>311</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>2026-09-14 14:57:10</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SP2-001778+SP2-001779</t>
+          <t>SP2-001753</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>832</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>DC2609220002</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="E38" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>DC2609220002</t>
-        </is>
-      </c>
-      <c r="Q38" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="R38" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 832</t>
+        <v>390</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>2609141KA8DDEA</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>CP2609140012</t>
+        </is>
+      </c>
+      <c r="M38" t="n">
+        <v>390</v>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>2026-09-14 15:05:24</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SP2-001607+SP2-001754</t>
+          <t>SP2-001755</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>794</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>DC2609220002</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="E39" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>DC2609220002</t>
-        </is>
-      </c>
-      <c r="Q39" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="R39" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 794</t>
+        <v>594</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>2609141KA8DDEA</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>CP2609140012</t>
+        </is>
+      </c>
+      <c r="M39" t="n">
+        <v>594</v>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>2026-09-14 15:05:24</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>PR5-000661</t>
+          <t>MNL-002435</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>8602</v>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>CP2609220002</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="n">
-        <v>46288</v>
-      </c>
-      <c r="E40" s="3" t="n">
-        <v>46304</v>
-      </c>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>CP2609220002</t>
-        </is>
-      </c>
-      <c r="Q40" s="3" t="n">
-        <v>46288</v>
-      </c>
-      <c r="R40" s="3" t="n">
-        <v>46304</v>
-      </c>
-      <c r="S40" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ก.ย. ราคา 8602</t>
+        <v>2737</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>2609251AWCE1CK</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>CP2609160013 DC2608280030</t>
+        </is>
+      </c>
+      <c r="M40" t="n">
+        <v>2737</v>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:59:46</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>OC</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SP1-001445+SP1-001446+SP1-001447+SP1-001448</t>
+          <t>SP1-001567+SP1-001568+SP1-001569+SP1-001570</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>11997</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>CP2609220007</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="E41" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="P41" t="inlineStr">
-        <is>
-          <t>CP2609220007</t>
-        </is>
-      </c>
-      <c r="Q41" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="R41" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="S41" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 11997</t>
-        </is>
+        <v>9036</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SP2-001803+SP2-001804+SP2-001805+SP2-001806</t>
+          <t>SP2-001858+SP2-001859</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2931</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>CP2609220002</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="E42" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>CP2609220002</t>
-        </is>
-      </c>
-      <c r="Q42" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="R42" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="S42" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 2931</t>
-        </is>
+        <v>1820</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SP2-001610+SP2-001611+SP2-001612+SP2-001613</t>
+          <t>SP4-000302</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1234</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>CP2609220007</t>
-        </is>
+        <v>141</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46288.00001157408</v>
+        <v>46288</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>46304.99998842592</v>
+        <v>46304</v>
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
-        </is>
-      </c>
-      <c r="Q43" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="R43" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="S43" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1234</t>
+          <t>DC2609220006</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
+          <t>SP2-001869+SP2-001870</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>950</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>CP2609220002</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="E44" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>CP2609220002</t>
-        </is>
-      </c>
-      <c r="Q44" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="R44" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="S44" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 950</t>
-        </is>
+        <v>903</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SP2-001753+SP2-001755</t>
+          <t>SP2-001749+SP2-001615+SP2-001616+SP2-001617</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1017</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>CP2609220007</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="E45" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>260930DC4DT2CY</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>CP2609220007</t>
-        </is>
-      </c>
-      <c r="M45" t="n">
-        <v>1017</v>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>2026-10-02 16:00:19</t>
-        </is>
-      </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>CP</t>
-        </is>
-      </c>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t>CP2609220007</t>
-        </is>
-      </c>
-      <c r="Q45" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="R45" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="S45" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1017</t>
-        </is>
+        <v>1241</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+          <t>SP2-001858+SP2-001859</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>955</v>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>CP2609220002</t>
-        </is>
+        <v>1861</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46288.00001157408</v>
+        <v>46279</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>260930DWC0FFR9</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>CP2609220002</t>
-        </is>
-      </c>
-      <c r="M46" t="n">
-        <v>955</v>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>2026-10-02 16:18:21</t>
-        </is>
-      </c>
-      <c r="O46" t="inlineStr">
-        <is>
-          <t>CP</t>
-        </is>
+        <v>46295</v>
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
-        </is>
-      </c>
-      <c r="Q46" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="R46" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="S46" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 955</t>
+          <t>DC2608310029 DC2609140003</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
+          <t>SP2-001778+SP2-001779</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1449</v>
+        <v>832</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
+          <t>DC2609220002</t>
         </is>
       </c>
       <c r="D47" s="3" t="n">
@@ -2236,32 +2138,9 @@
       <c r="E47" s="3" t="n">
         <v>46304.99998842592</v>
       </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>2609287HFYKV3U</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>CP2609220007</t>
-        </is>
-      </c>
-      <c r="M47" t="n">
-        <v>1449</v>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>2026-10-02 15:52:56</t>
-        </is>
-      </c>
-      <c r="O47" t="inlineStr">
-        <is>
-          <t>CP</t>
-        </is>
-      </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
+          <t>DC2609220002</t>
         </is>
       </c>
       <c r="Q47" s="3" t="n">
@@ -2272,18 +2151,18 @@
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1449</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 832</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SP1-001113</t>
+          <t>SP2-001607+SP2-001754</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1566</v>
+        <v>794</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -2291,63 +2170,40 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46288</v>
+        <v>46288.00001157408</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>46304</v>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>2609288A3EJJGE</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
+        <v>46304.99998842592</v>
+      </c>
+      <c r="P48" t="inlineStr">
         <is>
           <t>DC2609220002</t>
         </is>
       </c>
-      <c r="M48" t="n">
-        <v>1566</v>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>2026-10-02 16:15:10</t>
-        </is>
-      </c>
-      <c r="O48" t="inlineStr">
-        <is>
-          <t>CP</t>
-        </is>
-      </c>
-      <c r="P48" t="inlineStr">
-        <is>
-          <t>DC2609220002</t>
-        </is>
-      </c>
       <c r="Q48" s="3" t="n">
-        <v>46288</v>
+        <v>46288.00001157408</v>
       </c>
       <c r="R48" s="3" t="n">
-        <v>46304</v>
+        <v>46304.99998842592</v>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคา 1566</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 794</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SP1-001210</t>
+          <t>PR5-000661</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1412</v>
+        <v>8602</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>DC2609220002</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="D49" s="3" t="n">
@@ -2356,32 +2212,9 @@
       <c r="E49" s="3" t="n">
         <v>46304</v>
       </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>260929AW9BRK4J</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>DC2609220002</t>
-        </is>
-      </c>
-      <c r="M49" t="n">
-        <v>1412</v>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>2026-10-02 16:15:43</t>
-        </is>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>CP</t>
-        </is>
-      </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>DC2609220002</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="Q49" s="3" t="n">
@@ -2392,110 +2225,96 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคา 1412</t>
+          <t>Shp/TT เดือน ก.ย. ราคา 8602</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SP4-000241</t>
+          <t>SP1-001445+SP1-001446+SP1-001447+SP1-001448</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>400</v>
+        <v>11997</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>DC2608280023</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46266</v>
+        <v>46288.00001157408</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>46304</v>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>260929BD1UJHCV</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>DC2608280023</t>
-        </is>
-      </c>
-      <c r="M50" t="n">
-        <v>400</v>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>2026-10-02 16:35:35</t>
-        </is>
-      </c>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>CP</t>
-        </is>
+        <v>46304.99998842592</v>
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>DC2608280023</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="Q50" s="3" t="n">
-        <v>46266</v>
+        <v>46288.00001157408</v>
       </c>
       <c r="R50" s="3" t="n">
-        <v>46304</v>
+        <v>46304.99998842592</v>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>Shp Lzd TT ราคา400</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 11997</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SP4-000076</t>
+          <t>SP2-001803+SP2-001804+SP2-001805+SP2-001806</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>640</v>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>2610071JEP9U3K</t>
-        </is>
-      </c>
-      <c r="M51" t="n">
-        <v>590</v>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>2026-10-08 10:54:25</t>
-        </is>
-      </c>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>OC</t>
+        <v>2931</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>CP2609220002</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>46304.99998842592</v>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>CP2609220002</t>
+        </is>
+      </c>
+      <c r="Q51" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="R51" s="3" t="n">
+        <v>46304.99998842592</v>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 2931</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
+          <t>SP2-001610+SP2-001611+SP2-001612+SP2-001613</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>9551</v>
+        <v>1234</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="D52" s="3" t="n">
@@ -2504,32 +2323,9 @@
       <c r="E52" s="3" t="n">
         <v>46304.99998842592</v>
       </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>260930D84RADEG</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>CP2609220002</t>
-        </is>
-      </c>
-      <c r="M52" t="n">
-        <v>9551</v>
-      </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>2026-10-02 16:17:19</t>
-        </is>
-      </c>
-      <c r="O52" t="inlineStr">
-        <is>
-          <t>CP</t>
-        </is>
-      </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="Q52" s="3" t="n">
@@ -2540,22 +2336,22 @@
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 9551</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1234</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
+          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1199</v>
+        <v>950</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>DC2609220006</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="D53" s="3" t="n">
@@ -2564,32 +2360,9 @@
       <c r="E53" s="3" t="n">
         <v>46304.99998842592</v>
       </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>260930DWC0FFR9</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>DC2609220006</t>
-        </is>
-      </c>
-      <c r="M53" t="n">
-        <v>1199</v>
-      </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>2026-10-02 16:18:21</t>
-        </is>
-      </c>
-      <c r="O53" t="inlineStr">
-        <is>
-          <t>CP</t>
-        </is>
-      </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>DC2609220006</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="Q53" s="3" t="n">
@@ -2600,145 +2373,226 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1199</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 950</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MS2-000754</t>
+          <t>SP2-001753+SP2-001755</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>375</v>
+        <v>1017</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>CP2609220007</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>46304.99998842592</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>260929BD1UJHCV</t>
+          <t>260930DC4DT2CY</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>CP2609290069 DC2609290002</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="M54" t="n">
-        <v>375</v>
+        <v>1017</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>2026-10-02 16:35:35</t>
+          <t>2026-10-02 16:00:19</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>OC</t>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>CP2609220007</t>
+        </is>
+      </c>
+      <c r="Q54" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="R54" s="3" t="n">
+        <v>46304.99998842592</v>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1017</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>MS2-000820</t>
+          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>225</v>
+        <v>955</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CP2609220002</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>46304.99998842592</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>260929BD1UJHCV</t>
+          <t>260930DWC0FFR9</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>CP2609290069 DC2609290002</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="M55" t="n">
-        <v>225</v>
+        <v>955</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>2026-10-02 16:35:35</t>
+          <t>2026-10-02 16:18:21</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>CP2609220002</t>
+        </is>
+      </c>
+      <c r="Q55" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="R55" s="3" t="n">
+        <v>46304.99998842592</v>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 955</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>MS2-000942</t>
+          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>450</v>
+        <v>1449</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>CP2609220007</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>46304.99998842592</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>260929BD1UJHCV</t>
+          <t>2609287HFYKV3U</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>CP2609290069 DC2609290002</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="M56" t="n">
-        <v>450</v>
+        <v>1449</v>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>2026-10-02 16:35:35</t>
+          <t>2026-10-02 15:52:56</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>CP2609220007</t>
+        </is>
+      </c>
+      <c r="Q56" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="R56" s="3" t="n">
+        <v>46304.99998842592</v>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1449</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
+          <t>SP1-001113</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>9673</v>
+        <v>1566</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>CP2609090005</t>
+          <t>DC2609220002</t>
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46274.00001157408</v>
+        <v>46288</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>46303.99998842592</v>
+        <v>46304</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>261001FNX3QHKT</t>
+          <t>2609288A3EJJGE</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>CP2609090005</t>
+          <t>DC2609220002</t>
         </is>
       </c>
       <c r="M57" t="n">
-        <v>9673</v>
+        <v>1566</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>2026-10-02 17:47:09</t>
+          <t>2026-10-02 16:15:10</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
@@ -2748,116 +2602,746 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>CP2609090005</t>
+          <t>DC2609220002</t>
         </is>
       </c>
       <c r="Q57" s="3" t="n">
-        <v>46274.00001157408</v>
+        <v>46288</v>
       </c>
       <c r="R57" s="3" t="n">
-        <v>46303.99998842592</v>
+        <v>46304</v>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>Dynamic ก.ย. Shp ราคา 9673</t>
+          <t>Shp/TT เดือน ก.ย. ราคา 1566</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>MNL-002445</t>
+          <t>SP1-001210</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>2847</v>
+        <v>1412</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>DC2609220002</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E58" s="3" t="n">
+        <v>46304</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>261001FVHQUH0S</t>
+          <t>260929AW9BRK4J</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>CP2609280021 DC2609280008</t>
+          <t>DC2609220002</t>
         </is>
       </c>
       <c r="M58" t="n">
-        <v>2847</v>
+        <v>1412</v>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>2026-10-02 16:32:59</t>
+          <t>2026-10-02 16:15:43</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>OC</t>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>DC2609220002</t>
+        </is>
+      </c>
+      <c r="Q58" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="R58" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคา 1412</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>SP4-000241</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>400</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>DC2608280023</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46031</v>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>46275</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>260929BD1UJHCV</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>DC2608280023</t>
+        </is>
+      </c>
+      <c r="M59" t="n">
+        <v>400</v>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:35:35</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>DC2608280023</t>
+        </is>
+      </c>
+      <c r="Q59" s="3" t="n">
+        <v>46031</v>
+      </c>
+      <c r="R59" s="3" t="n">
+        <v>46275</v>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>Shp Lzd TT ราคา400</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>SP4-000076</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>640</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>2610071JEP9U3K</t>
+        </is>
+      </c>
+      <c r="M60" t="n">
+        <v>590</v>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>2026-10-08 10:54:25</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>OC</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>9551</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>CP2609220002</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>46304.99998842592</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>260930D84RADEG</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>CP2609220002</t>
+        </is>
+      </c>
+      <c r="M61" t="n">
+        <v>9551</v>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:17:19</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>CP2609220002</t>
+        </is>
+      </c>
+      <c r="Q61" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="R61" s="3" t="n">
+        <v>46304.99998842592</v>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 9551</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>1199</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>DC2609220006</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>46304.99998842592</v>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>260930DWC0FFR9</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>DC2609220006</t>
+        </is>
+      </c>
+      <c r="M62" t="n">
+        <v>1199</v>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:18:21</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>DC2609220006</t>
+        </is>
+      </c>
+      <c r="Q62" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="R62" s="3" t="n">
+        <v>46304.99998842592</v>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1199</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>MS2-000754</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>375</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>260929BD1UJHCV</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>CP2609290069 DC2609290002</t>
+        </is>
+      </c>
+      <c r="M63" t="n">
+        <v>375</v>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:35:35</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>OC</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>MS2-000820</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>225</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>260929BD1UJHCV</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>CP2609290069 DC2609290002</t>
+        </is>
+      </c>
+      <c r="M64" t="n">
+        <v>225</v>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:35:35</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>MS2-000942</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>450</v>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>260929BD1UJHCV</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>CP2609290069 DC2609290002</t>
+        </is>
+      </c>
+      <c r="M65" t="n">
+        <v>450</v>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:35:35</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>9673</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>CP2609090005</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46274.00001157408</v>
+      </c>
+      <c r="E66" s="3" t="n">
+        <v>46303.99998842592</v>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>261001FNX3QHKT</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>CP2609090005</t>
+        </is>
+      </c>
+      <c r="M66" t="n">
+        <v>9673</v>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>2026-10-02 17:47:09</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>CP2609090005</t>
+        </is>
+      </c>
+      <c r="Q66" s="3" t="n">
+        <v>46274.00001157408</v>
+      </c>
+      <c r="R66" s="3" t="n">
+        <v>46303.99998842592</v>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>Dynamic ก.ย. Shp ราคา 9673</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>MNL-002445</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>2847</v>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>261001FVHQUH0S</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>CP2609280021 DC2609280008</t>
+        </is>
+      </c>
+      <c r="M67" t="n">
+        <v>2847</v>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:32:59</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>OC</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
           <t>SP1-001113</t>
         </is>
       </c>
-      <c r="B59" t="n">
+      <c r="B68" t="n">
         <v>1603</v>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t>DC2609290041</t>
         </is>
       </c>
-      <c r="D59" s="3" t="n">
+      <c r="D68" s="3" t="n">
+        <v>46032</v>
+      </c>
+      <c r="E68" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>261002HSH1MCYP</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="M68" t="n">
+        <v>1603</v>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>2026-10-02 18:00:21</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="Q68" s="3" t="n">
+        <v>46032</v>
+      </c>
+      <c r="R68" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 1603</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>SP1-001449</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>2220</v>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:05:23</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>DC2610010003</t>
+        </is>
+      </c>
+      <c r="Q69" s="3" t="n">
         <v>46296</v>
       </c>
-      <c r="E59" s="3" t="n">
-        <v>46326</v>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>261002HSH1MCYP</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
+      <c r="R69" s="3" t="n">
+        <v>46336</v>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>Shp+Lzd+Tiktok ราคา 2220</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>SP2-001778+SP2-001779</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>851</v>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:09:24</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
         <is>
           <t>DC2609290041</t>
         </is>
       </c>
-      <c r="M59" t="n">
-        <v>1603</v>
-      </c>
-      <c r="N59" t="inlineStr">
-        <is>
-          <t>2026-10-02 18:00:21</t>
-        </is>
-      </c>
-      <c r="O59" t="inlineStr">
+      <c r="Q70" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="R70" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 851</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>SP2-001607+SP2-001754</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>810</v>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:10:32</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="Q71" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="R71" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 810</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>MS2-000818</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>225</v>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>261007288HJTKT</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>CP2609290069 DC2609290002</t>
+        </is>
+      </c>
+      <c r="M72" t="n">
+        <v>225</v>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:12:30</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
         <is>
           <t>CP</t>
         </is>
       </c>
-      <c r="P59" t="inlineStr">
-        <is>
-          <t>DC2609290041</t>
-        </is>
-      </c>
-      <c r="Q59" s="3" t="n">
-        <v>46296</v>
-      </c>
-      <c r="R59" s="3" t="n">
-        <v>46326</v>
-      </c>
-      <c r="S59" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ต.ค. ราคา 1603</t>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>SP2-001753+SP2-001755</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>993</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>CP2610050027</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46152.00001157408</v>
+      </c>
+      <c r="E73" s="3" t="n">
+        <v>46315.99998842592</v>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:13:20</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>CP2610050027</t>
+        </is>
+      </c>
+      <c r="Q73" s="3" t="n">
+        <v>46152.00001157408</v>
+      </c>
+      <c r="R73" s="3" t="n">
+        <v>46315.99998842592</v>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>FS Shp ถูกชัวร์ ราคาเซ็ทละ 993</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>1052</v>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:16:15</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>CP2610060010</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>07/10/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>20/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>FS Shp ราคาเซ็ทละ 1052</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S59"/>
+  <autoFilter ref="A1:S74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(pricing_engine): prioritize combo coupon description over sub-sku detail remark and resolve remark conflict wipe
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/cp_data.xlsx
+++ b/projects/auto_page/autopageMKII/tables/cp_data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$S$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$S$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S74"/>
+  <dimension ref="A1:S76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -556,7 +556,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>261007265U804D</t>
+          <t>2610083HW7WMDS</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-10-08 11:11:26</t>
+          <t>2026-10-08 11:29:33</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -588,6 +588,11 @@
       <c r="R2" s="3" t="n">
         <v>46326.99998842592</v>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1056</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -611,7 +616,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2610071YKH3P16</t>
+          <t>2610082Q1FEJVD</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -624,7 +629,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-10-08 11:07:28</t>
+          <t>2026-10-08 11:23:58</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -712,39 +717,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SP4-000302</t>
+          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>139</v>
+        <v>974</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DC2609300024</t>
+          <t>CP2609290081</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46032</v>
+        <v>46296.00001157408</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>46326</v>
+        <v>46326.99998842592</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>261005SRV913UJ</t>
+          <t>2610082M7WMJXX</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>DC2609300024</t>
+          <t>CP2609290081</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>139</v>
+        <v>974</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-10-08 11:09:55</t>
+          <t>2026-10-08 11:22:03</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -754,33 +759,33 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>DC2609300024</t>
+          <t>CP2609290081</t>
         </is>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>46296</v>
+        <v>46296.00001157408</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>46326</v>
+        <v>46326.99998842592</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคา 139</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 974</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>974</v>
+        <v>1477</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
@@ -791,20 +796,20 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>26100729P4PHTQ</t>
+          <t>2610083CRKVQ58</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>974</v>
+        <v>1477</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-10-08 11:15:29</t>
+          <t>2026-10-08 11:28:37</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -814,7 +819,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="Q6" s="3" t="n">
@@ -825,77 +830,82 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 974</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1477</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SP2-001753+SP2-001755</t>
+          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>993</v>
+        <v>969</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CP2609140012</t>
+          <t>CP2609290081</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46279.00001157408</v>
+        <v>46296.00001157408</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>46304</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>5 4</t>
-        </is>
+        <v>46326.99998842592</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>261003K6J8B8H5</t>
+          <t>2610072A84PSC3</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>CP2609140012</t>
+          <t>CP2609290081</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>993</v>
+        <v>969</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-10-08 11:13:37</t>
+          <t>2026-10-08 11:18:01</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>CP + OC</t>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
         </is>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>46300.00001157408</v>
+        <v>46296.00001157408</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>46337.99998842592</v>
+        <v>46326.99998842592</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 969</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
+          <t>SP2-001748+SP2-001615+SP2-001616+SP2-001617</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1477</v>
+        <v>1330</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
+          <t>DC2609290042</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
@@ -906,20 +916,20 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2610071PP00HWD</t>
+          <t>26100704X2FT1A</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
+          <t>DC2609290042</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>1477</v>
+        <v>1330</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-10-08 11:00:07</t>
+          <t>2026-10-08 10:35:49</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -929,7 +939,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
+          <t>DC2609290042</t>
         </is>
       </c>
       <c r="Q8" s="3" t="n">
@@ -940,106 +950,74 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1477</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 1330</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
+          <t>SP4-000076</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>969</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CP2609290081</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>46296.00001157408</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>46326.99998842592</v>
+        <v>590</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2610072A0U120S</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>CP2609290081</t>
+          <t>2610071JEP9U3K</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>969</v>
+        <v>590</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-10-08 11:17:02</t>
+          <t>2026-10-08 10:54:25</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>CP</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>CP2609290081</t>
-        </is>
-      </c>
-      <c r="Q9" s="3" t="n">
-        <v>46296.00001157408</v>
-      </c>
-      <c r="R9" s="3" t="n">
-        <v>46326.99998842592</v>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 969</t>
+          <t>OC</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SP2-001748+SP2-001615+SP2-001616+SP2-001617</t>
+          <t>SP1-001378</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1330</v>
+        <v>3031</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DC2609290042</t>
+          <t>CP2609290081</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46296.00001157408</v>
+        <v>46296</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>46326.99998842592</v>
+        <v>46326</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>26100704X2FT1A</t>
+          <t>261005SB6KAGSA</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>DC2609290042</t>
+          <t>CP2609290081</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>1330</v>
+        <v>3031</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-10-08 10:35:49</t>
+          <t>2026-10-05 15:28:13</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1049,85 +1027,117 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>DC2609290042</t>
+          <t>CP2609290081</t>
         </is>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>46296.00001157408</v>
+        <v>46296</v>
       </c>
       <c r="R10" s="3" t="n">
-        <v>46326.99998842592</v>
+        <v>46326</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 1330</t>
+          <t>Shp/TT เดือน ต.ค. ราคา 3031</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SP4-000076</t>
+          <t>SP4-000241</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>590</v>
+        <v>405</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>DC2610010003</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>46336</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2610071JEP9U3K</t>
+          <t>261006V8F25WXF</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>DC2610010003</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>590</v>
+        <v>405</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-10-08 10:54:25</t>
+          <t>2026-10-08 10:34:53</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>OC</t>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>DC2610010003</t>
+        </is>
+      </c>
+      <c r="Q11" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R11" s="3" t="n">
+        <v>46336</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Shp+Lzd+Tiktok ราคา 405</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SP1-001378</t>
+          <t>SP4-000196</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3031</v>
+        <v>305</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>DC2609300024</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46296</v>
+        <v>46032</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>46326</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>261005SB6KAGSA</t>
+          <t>2610071NYB574H</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>DC2609300024</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>3031</v>
+        <v>305</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-10-05 15:28:13</t>
+          <t>2026-10-08 11:46:06</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1137,179 +1147,151 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>DC2609300024</t>
         </is>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>46296</v>
+        <v>46032</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>46326</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคา 3031</t>
+          <t>Shp/TT เดือน ต.ค. ราคา 305</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SP4-000241</t>
+          <t>TEST-PATTERN-SKU</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>405</v>
+        <v>999</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>DC2610010003</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>46296</v>
-      </c>
-      <c r="E13" s="3" t="n">
-        <v>46336</v>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>261006V8F25WXF</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>DC2610010003</t>
-        </is>
-      </c>
-      <c r="M13" t="n">
-        <v>405</v>
+          <t>CP_INSERTED</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-10-08 10:34:53</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>CP</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>DC2610010003</t>
-        </is>
-      </c>
-      <c r="Q13" s="3" t="n">
-        <v>46296</v>
-      </c>
-      <c r="R13" s="3" t="n">
-        <v>46336</v>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>Shp+Lzd+Tiktok ราคา 405</t>
+          <t>08/10/2026 11:09:23</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SP2-001799+SP2-001800+SP2-001801+SP2-001802</t>
+          <t>TEST-PATTERN-SKU-2</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1849</v>
+        <v>999</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CP_NEW</t>
+        </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-10-08 10:36:36</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>CP2609210010</t>
-        </is>
-      </c>
-      <c r="Q14" s="3" t="n">
-        <v>46286.00001157408</v>
-      </c>
-      <c r="R14" s="3" t="n">
-        <v>46303.99998842592</v>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>Dynamic ก.ย. Shp ราคาเซท 1849</t>
+          <t>08/10/2026 11:02:06</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+          <t>SP2-001869+SP2-001870</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>952</v>
+        <v>921</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2610071V2MM04F</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>921</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-10-08 10:41:56</t>
+          <t>2026-10-08 11:50:02</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>CP2610060006</t>
+          <t>DC2609290041</t>
         </is>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>46302.00001157408</v>
+        <v>46296.00001157408</v>
       </c>
       <c r="R15" s="3" t="n">
-        <v>46315.99998842592</v>
+        <v>46326.99998842592</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>FS Shp ราคาเซท 952</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 921</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SP4-000196</t>
+          <t>SP1-001449</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>305</v>
+        <v>2220</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>DC2609300024</t>
+          <t>DC2610010003</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46032</v>
+        <v>46296</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>46326</v>
+        <v>46336</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2610071MEQQ7CT</t>
+          <t>2610071VPKHFM4</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>DC2609300024</t>
+          <t>DC2610010003</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>305</v>
+        <v>2220</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-10-08 10:58:32</t>
+          <t>2026-10-08 11:50:32</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1319,534 +1301,561 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>DC2609300024</t>
+          <t>DC2610010003</t>
         </is>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>46032</v>
+        <v>46296</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>46326</v>
+        <v>46336</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคา 305</t>
+          <t>Shp+Lzd+Tiktok ราคา 2220</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SP2-001803+SP2-001804+SP2-001805+SP2-001806</t>
+          <t>TEST-PATTERN-SKU</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2993</v>
+        <v>888</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CP_NEW_PRICE</t>
+        </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-10-08 10:59:18</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>CP2609290081</t>
-        </is>
-      </c>
-      <c r="Q17" s="3" t="n">
-        <v>46296.00001157408</v>
-      </c>
-      <c r="R17" s="3" t="n">
-        <v>46326.99998842592</v>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 2993</t>
+          <t>08/10/2026 11:06:56</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TEST-PATTERN-SKU</t>
+          <t>SP2-001778+SP2-001779</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>999</v>
+        <v>851</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CP_INSERTED</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>26100839JAVCJ8</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>851</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>08/10/2026 11:09:23</t>
+          <t>2026-10-08 11:26:00</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="R18" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 851</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TEST-PATTERN-SKU-2</t>
+          <t>SP2-001607+SP2-001754</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>999</v>
+        <v>810</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CP_NEW</t>
-        </is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2610072GWE2YKY</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>810</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>08/10/2026 11:02:06</t>
+          <t>2026-10-08 11:19:24</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="Q19" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="R19" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 810</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SP2-001869+SP2-001870</t>
+          <t>MS2-000818</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>921</v>
+        <v>225</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CP2609290069 DC2609290002</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>261007288HJTKT</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>CP2609290069 DC2609290002</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>225</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-10-08 11:04:54</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>DC2609290041</t>
-        </is>
-      </c>
-      <c r="Q20" s="3" t="n">
-        <v>46296.00001157408</v>
-      </c>
-      <c r="R20" s="3" t="n">
-        <v>46326.99998842592</v>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 921</t>
+          <t>2026-10-08 11:12:30</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SP1-001449</t>
+          <t>SP4-000302</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2220</v>
+        <v>137</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DC2610010003</t>
+          <t>DC2608210007</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46296</v>
+        <v>46258</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>46336</v>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>2026-10-08 11:05:23</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>DC2610010003</t>
-        </is>
-      </c>
-      <c r="Q21" s="3" t="n">
-        <v>46296</v>
-      </c>
-      <c r="R21" s="3" t="n">
-        <v>46336</v>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>Shp+Lzd+Tiktok ราคา 2220</t>
-        </is>
+        <v>46273</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TEST-PATTERN-SKU</t>
+          <t>SP4-000242</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>888</v>
+        <v>860</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CP_NEW_PRICE</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>08/10/2026 11:06:56</t>
-        </is>
+          <t>DC2607310017</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>46235</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>46273</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SP2-001778+SP2-001779</t>
+          <t>SP4-000302</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>851</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>DC2609290041</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>46296.00001157408</v>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>46326.99998842592</v>
+        <v>143</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>2609141SRMKUEH</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>DC2609140005</t>
+        </is>
+      </c>
+      <c r="M23" t="n">
+        <v>141</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-10-08 11:09:24</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>DC2609290041</t>
-        </is>
-      </c>
-      <c r="Q23" s="3" t="n">
-        <v>46296.00001157408</v>
-      </c>
-      <c r="R23" s="3" t="n">
-        <v>46326.99998842592</v>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 851</t>
+          <t>2026-09-14 14:53:23</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SP2-001607+SP2-001754</t>
+          <t>SP2-001713</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>810</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>DC2609290041</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="n">
-        <v>46296.00001157408</v>
-      </c>
-      <c r="E24" s="3" t="n">
-        <v>46326.99998842592</v>
+        <v>300</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>2609141MCF7RSD</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>DC2609140005</t>
+        </is>
+      </c>
+      <c r="M24" t="n">
+        <v>300</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-10-08 11:10:32</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>DC2609290041</t>
-        </is>
-      </c>
-      <c r="Q24" s="3" t="n">
-        <v>46296.00001157408</v>
-      </c>
-      <c r="R24" s="3" t="n">
-        <v>46326.99998842592</v>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 810</t>
+          <t>2026-09-14 14:48:42</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MS2-000818</t>
+          <t>SP2-001714</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>225</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>CP2609290069 DC2609290002</t>
-        </is>
+        <v>300</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>261007288HJTKT</t>
+          <t>2609141MCF7RSD</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>CP2609290069 DC2609290002</t>
+          <t>DC2609140005</t>
         </is>
       </c>
       <c r="M25" t="n">
-        <v>225</v>
+        <v>300</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-10-08 11:12:30</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>CP</t>
+          <t>2026-09-14 14:48:42</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SP4-000302</t>
+          <t>SP2-001715</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>137</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>DC2608210007</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>46258</v>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>46273</v>
+        <v>301</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>2609141MCF7RSD</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>DC2609140005</t>
+        </is>
+      </c>
+      <c r="M26" t="n">
+        <v>301</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>2026-09-14 14:48:42</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SP4-000242</t>
+          <t>SP2-001716</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>860</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>DC2607310017</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="n">
-        <v>46235</v>
-      </c>
-      <c r="E27" s="3" t="n">
-        <v>46273</v>
+        <v>301</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>2609141MCF7RSD</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>DC2609140005</t>
+        </is>
+      </c>
+      <c r="M27" t="n">
+        <v>301</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>2026-09-14 14:48:42</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SP4-000302</t>
+          <t>SP1-001579</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>143</v>
+        <v>1404</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>2609141SRMKUEH</t>
+          <t>2609141P1CYP3G</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>DC2609140005</t>
+          <t>DC2609140008</t>
         </is>
       </c>
       <c r="M28" t="n">
-        <v>141</v>
+        <v>1404</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-09-14 14:53:23</t>
+          <t>2026-09-14 14:51:36</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SP2-001713</t>
+          <t>SP2-001610</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>300</v>
+        <v>311</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2609141MCF7RSD</t>
+          <t>2609141P4RQJXW</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>DC2609140005</t>
+          <t>CP2609140012</t>
         </is>
       </c>
       <c r="M29" t="n">
-        <v>300</v>
+        <v>311</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-09-14 14:48:42</t>
+          <t>2026-09-14 14:57:10</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SP2-001714</t>
+          <t>SP2-001611</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2609141MCF7RSD</t>
+          <t>2609141P4RQJXW</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>DC2609140005</t>
+          <t>CP2609140012</t>
         </is>
       </c>
       <c r="M30" t="n">
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-09-14 14:48:42</t>
+          <t>2026-09-14 14:57:10</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SP2-001715</t>
+          <t>SP2-001612</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2609141MCF7RSD</t>
+          <t>2609141P4RQJXW</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>DC2609140005</t>
+          <t>CP2609140012</t>
         </is>
       </c>
       <c r="M31" t="n">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-09-14 14:48:42</t>
+          <t>2026-09-14 14:57:10</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SP2-001716</t>
+          <t>SP2-001613</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>301</v>
+        <v>311</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2609141MCF7RSD</t>
+          <t>2609141P4RQJXW</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>DC2609140005</t>
+          <t>CP2609140012</t>
         </is>
       </c>
       <c r="M32" t="n">
-        <v>301</v>
+        <v>311</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-09-14 14:48:42</t>
+          <t>2026-09-14 14:57:10</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SP1-001579</t>
+          <t>SP2-001753</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1404</v>
+        <v>390</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2609141P1CYP3G</t>
+          <t>2609141KA8DDEA</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>DC2609140008</t>
+          <t>CP2609140012</t>
         </is>
       </c>
       <c r="M33" t="n">
-        <v>1404</v>
+        <v>390</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-09-14 14:51:36</t>
+          <t>2026-09-14 15:05:24</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SP2-001610</t>
+          <t>SP2-001755</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>311</v>
+        <v>594</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2609141P4RQJXW</t>
+          <t>2609141KA8DDEA</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -1855,281 +1864,325 @@
         </is>
       </c>
       <c r="M34" t="n">
-        <v>311</v>
+        <v>594</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-09-14 14:57:10</t>
+          <t>2026-09-14 15:05:24</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SP2-001611</t>
+          <t>MNL-002435</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>310</v>
+        <v>2737</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2609141P4RQJXW</t>
+          <t>2609251AWCE1CK</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>CP2609140012</t>
+          <t>CP2609160013 DC2608280030</t>
         </is>
       </c>
       <c r="M35" t="n">
-        <v>310</v>
+        <v>2737</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-09-14 14:57:10</t>
+          <t>2026-09-29 14:59:46</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>OC</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SP2-001612</t>
+          <t>SP1-001567+SP1-001568+SP1-001569+SP1-001570</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>310</v>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>2609141P4RQJXW</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>CP2609140012</t>
-        </is>
-      </c>
-      <c r="M36" t="n">
-        <v>310</v>
-      </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>2026-09-14 14:57:10</t>
-        </is>
+        <v>9036</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SP2-001613</t>
+          <t>SP2-001858+SP2-001859</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>311</v>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>2609141P4RQJXW</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>CP2609140012</t>
-        </is>
-      </c>
-      <c r="M37" t="n">
-        <v>311</v>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>2026-09-14 14:57:10</t>
-        </is>
+        <v>1820</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SP2-001753</t>
+          <t>SP4-000302</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>390</v>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>2609141KA8DDEA</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>CP2609140012</t>
-        </is>
-      </c>
-      <c r="M38" t="n">
-        <v>390</v>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>2026-09-14 15:05:24</t>
+        <v>141</v>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>DC2609220006</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SP2-001755</t>
+          <t>SP2-001869+SP2-001870</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>594</v>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>2609141KA8DDEA</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>CP2609140012</t>
-        </is>
-      </c>
-      <c r="M39" t="n">
-        <v>594</v>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>2026-09-14 15:05:24</t>
-        </is>
+        <v>903</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MNL-002435</t>
+          <t>SP2-001749+SP2-001615+SP2-001616+SP2-001617</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2737</v>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>2609251AWCE1CK</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>CP2609160013 DC2608280030</t>
-        </is>
-      </c>
-      <c r="M40" t="n">
-        <v>2737</v>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>2026-09-29 14:59:46</t>
-        </is>
-      </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>OC</t>
-        </is>
+        <v>1241</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SP1-001567+SP1-001568+SP1-001569+SP1-001570</t>
+          <t>SP2-001858+SP2-001859</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>9036</v>
+        <v>1861</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>DC2608310029 DC2609140003</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>DC2608310029 DC2609140003</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SP2-001858+SP2-001859</t>
+          <t>SP2-001778+SP2-001779</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1820</v>
+        <v>832</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>DC2609220002</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>46304.99998842592</v>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>DC2609220002</t>
+        </is>
+      </c>
+      <c r="Q42" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="R42" s="3" t="n">
+        <v>46304.99998842592</v>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 832</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SP4-000302</t>
+          <t>SP2-001607+SP2-001754</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>141</v>
+        <v>794</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>DC2609220002</t>
+        </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46288</v>
+        <v>46288.00001157408</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>46304</v>
+        <v>46304.99998842592</v>
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>DC2609220006</t>
+          <t>DC2609220002</t>
+        </is>
+      </c>
+      <c r="Q43" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="R43" s="3" t="n">
+        <v>46304.99998842592</v>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 794</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SP2-001869+SP2-001870</t>
+          <t>PR5-000661</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>903</v>
+        <v>8602</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>CP2609220002</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>CP2609220002</t>
+        </is>
+      </c>
+      <c r="Q44" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="R44" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคา 8602</t>
+        </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SP2-001749+SP2-001615+SP2-001616+SP2-001617</t>
+          <t>SP1-001445+SP1-001446+SP1-001447+SP1-001448</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1241</v>
+        <v>11997</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CP2609220007</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>46304.99998842592</v>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>CP2609220007</t>
+        </is>
+      </c>
+      <c r="Q45" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="R45" s="3" t="n">
+        <v>46304.99998842592</v>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 11997</t>
+        </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SP2-001858+SP2-001859</t>
+          <t>SP2-001803+SP2-001804+SP2-001805+SP2-001806</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1861</v>
+        <v>2931</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>CP2609220002</t>
+        </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46279</v>
+        <v>46288.00001157408</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>46295</v>
+        <v>46304.99998842592</v>
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>DC2608310029 DC2609140003</t>
+          <t>CP2609220002</t>
+        </is>
+      </c>
+      <c r="Q46" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="R46" s="3" t="n">
+        <v>46304.99998842592</v>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 2931</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SP2-001778+SP2-001779</t>
+          <t>SP2-001610+SP2-001611+SP2-001612+SP2-001613</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>832</v>
+        <v>1234</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>DC2609220002</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="D47" s="3" t="n">
@@ -2140,7 +2193,7 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>DC2609220002</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="Q47" s="3" t="n">
@@ -2151,22 +2204,22 @@
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 832</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1234</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SP2-001607+SP2-001754</t>
+          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>794</v>
+        <v>950</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>DC2609220002</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="D48" s="3" t="n">
@@ -2177,7 +2230,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>DC2609220002</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="Q48" s="3" t="n">
@@ -2188,59 +2241,82 @@
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 794</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 950</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PR5-000661</t>
+          <t>SP2-001753+SP2-001755</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>8602</v>
+        <v>1017</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46288</v>
+        <v>46288.00001157408</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>46304</v>
+        <v>46304.99998842592</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>260930DC4DT2CY</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>CP2609220007</t>
+        </is>
+      </c>
+      <c r="M49" t="n">
+        <v>1017</v>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:00:19</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="Q49" s="3" t="n">
-        <v>46288</v>
+        <v>46288.00001157408</v>
       </c>
       <c r="R49" s="3" t="n">
-        <v>46304</v>
+        <v>46304.99998842592</v>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคา 8602</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1017</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SP1-001445+SP1-001446+SP1-001447+SP1-001448</t>
+          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>11997</v>
+        <v>955</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="D50" s="3" t="n">
@@ -2249,9 +2325,32 @@
       <c r="E50" s="3" t="n">
         <v>46304.99998842592</v>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>260930DWC0FFR9</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>CP2609220002</t>
+        </is>
+      </c>
+      <c r="M50" t="n">
+        <v>955</v>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:18:21</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="Q50" s="3" t="n">
@@ -2262,22 +2361,22 @@
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 11997</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 955</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SP2-001803+SP2-001804+SP2-001805+SP2-001806</t>
+          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>2931</v>
+        <v>1449</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="D51" s="3" t="n">
@@ -2286,9 +2385,32 @@
       <c r="E51" s="3" t="n">
         <v>46304.99998842592</v>
       </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>2609287HFYKV3U</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>CP2609220007</t>
+        </is>
+      </c>
+      <c r="M51" t="n">
+        <v>1449</v>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:52:56</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
+          <t>CP2609220007</t>
         </is>
       </c>
       <c r="Q51" s="3" t="n">
@@ -2299,120 +2421,166 @@
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 2931</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1449</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SP2-001610+SP2-001611+SP2-001612+SP2-001613</t>
+          <t>SP1-001113</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1234</v>
+        <v>1566</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
+          <t>DC2609220002</t>
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46288.00001157408</v>
+        <v>46288</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>46304.99998842592</v>
+        <v>46304</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>2609288A3EJJGE</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>DC2609220002</t>
+        </is>
+      </c>
+      <c r="M52" t="n">
+        <v>1566</v>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:15:10</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
+          <t>DC2609220002</t>
         </is>
       </c>
       <c r="Q52" s="3" t="n">
-        <v>46288.00001157408</v>
+        <v>46288</v>
       </c>
       <c r="R52" s="3" t="n">
-        <v>46304.99998842592</v>
+        <v>46304</v>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1234</t>
+          <t>Shp/TT เดือน ก.ย. ราคา 1566</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
+          <t>SP1-001210</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>950</v>
+        <v>1412</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
+          <t>DC2609220002</t>
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46288.00001157408</v>
+        <v>46288</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>46304.99998842592</v>
+        <v>46304</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>260929AW9BRK4J</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>DC2609220002</t>
+        </is>
+      </c>
+      <c r="M53" t="n">
+        <v>1412</v>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:15:43</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
+          <t>DC2609220002</t>
         </is>
       </c>
       <c r="Q53" s="3" t="n">
-        <v>46288.00001157408</v>
+        <v>46288</v>
       </c>
       <c r="R53" s="3" t="n">
-        <v>46304.99998842592</v>
+        <v>46304</v>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 950</t>
+          <t>Shp/TT เดือน ก.ย. ราคา 1412</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SP2-001753+SP2-001755</t>
+          <t>SP4-000241</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1017</v>
+        <v>400</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
+          <t>DC2608280023</t>
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46288.00001157408</v>
+        <v>46031</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>46304.99998842592</v>
+        <v>46275</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>260930DC4DT2CY</t>
+          <t>260929BD1UJHCV</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
+          <t>DC2608280023</t>
         </is>
       </c>
       <c r="M54" t="n">
-        <v>1017</v>
+        <v>400</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>2026-10-02 16:00:19</t>
+          <t>2026-10-02 16:35:35</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
@@ -2422,93 +2590,61 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
+          <t>DC2608280023</t>
         </is>
       </c>
       <c r="Q54" s="3" t="n">
-        <v>46288.00001157408</v>
+        <v>46031</v>
       </c>
       <c r="R54" s="3" t="n">
-        <v>46304.99998842592</v>
+        <v>46275</v>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1017</t>
+          <t>Shp Lzd TT ราคา400</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+          <t>SP4-000076</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>955</v>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>CP2609220002</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="E55" s="3" t="n">
-        <v>46304.99998842592</v>
+        <v>640</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>260930DWC0FFR9</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>CP2609220002</t>
+          <t>2610071JEP9U3K</t>
         </is>
       </c>
       <c r="M55" t="n">
-        <v>955</v>
+        <v>590</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>2026-10-02 16:18:21</t>
+          <t>2026-10-08 10:54:25</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>CP</t>
-        </is>
-      </c>
-      <c r="P55" t="inlineStr">
-        <is>
-          <t>CP2609220002</t>
-        </is>
-      </c>
-      <c r="Q55" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="R55" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="S55" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 955</t>
+          <t>OC</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
+          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1449</v>
+        <v>9551</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="D56" s="3" t="n">
@@ -2519,20 +2655,20 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>2609287HFYKV3U</t>
+          <t>260930D84RADEG</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="M56" t="n">
-        <v>1449</v>
+        <v>9551</v>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>2026-10-02 15:52:56</t>
+          <t>2026-10-02 16:17:19</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
@@ -2542,7 +2678,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>CP2609220007</t>
+          <t>CP2609220002</t>
         </is>
       </c>
       <c r="Q56" s="3" t="n">
@@ -2553,46 +2689,46 @@
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1449</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซท 9551</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SP1-001113</t>
+          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1566</v>
+        <v>1199</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>DC2609220002</t>
+          <t>DC2609220006</t>
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46288</v>
+        <v>46288.00001157408</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>46304</v>
+        <v>46304.99998842592</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>2609288A3EJJGE</t>
+          <t>260930DWC0FFR9</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>DC2609220002</t>
+          <t>DC2609220006</t>
         </is>
       </c>
       <c r="M57" t="n">
-        <v>1566</v>
+        <v>1199</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>2026-10-02 16:15:10</t>
+          <t>2026-10-02 16:18:21</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
@@ -2602,100 +2738,62 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>DC2609220002</t>
+          <t>DC2609220006</t>
         </is>
       </c>
       <c r="Q57" s="3" t="n">
-        <v>46288</v>
+        <v>46288.00001157408</v>
       </c>
       <c r="R57" s="3" t="n">
-        <v>46304</v>
+        <v>46304.99998842592</v>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคา 1566</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1199</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SP1-001210</t>
+          <t>MS2-000754</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>1412</v>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>DC2609220002</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="n">
-        <v>46288</v>
-      </c>
-      <c r="E58" s="3" t="n">
-        <v>46304</v>
+        <v>375</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>260929AW9BRK4J</t>
+          <t>260929BD1UJHCV</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>DC2609220002</t>
+          <t>CP2609290069 DC2609290002</t>
         </is>
       </c>
       <c r="M58" t="n">
-        <v>1412</v>
+        <v>375</v>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>2026-10-02 16:15:43</t>
+          <t>2026-10-02 16:35:35</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>CP</t>
-        </is>
-      </c>
-      <c r="P58" t="inlineStr">
-        <is>
-          <t>DC2609220002</t>
-        </is>
-      </c>
-      <c r="Q58" s="3" t="n">
-        <v>46288</v>
-      </c>
-      <c r="R58" s="3" t="n">
-        <v>46304</v>
-      </c>
-      <c r="S58" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ก.ย. ราคา 1412</t>
+          <t>OC</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SP4-000241</t>
+          <t>MS2-000820</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>400</v>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>DC2608280023</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="n">
-        <v>46031</v>
-      </c>
-      <c r="E59" s="3" t="n">
-        <v>46275</v>
+        <v>225</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
@@ -2704,11 +2802,11 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>DC2608280023</t>
+          <t>CP2609290069 DC2609290002</t>
         </is>
       </c>
       <c r="M59" t="n">
-        <v>400</v>
+        <v>225</v>
       </c>
       <c r="N59" t="inlineStr">
         <is>
@@ -2717,51 +2815,40 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>CP</t>
-        </is>
-      </c>
-      <c r="P59" t="inlineStr">
-        <is>
-          <t>DC2608280023</t>
-        </is>
-      </c>
-      <c r="Q59" s="3" t="n">
-        <v>46031</v>
-      </c>
-      <c r="R59" s="3" t="n">
-        <v>46275</v>
-      </c>
-      <c r="S59" t="inlineStr">
-        <is>
-          <t>Shp Lzd TT ราคา400</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>SP4-000076</t>
+          <t>MS2-000942</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>640</v>
+        <v>450</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>2610071JEP9U3K</t>
+          <t>260929BD1UJHCV</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>CP2609290069 DC2609290002</t>
         </is>
       </c>
       <c r="M60" t="n">
-        <v>590</v>
+        <v>450</v>
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>2026-10-08 10:54:25</t>
+          <t>2026-10-02 16:35:35</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>OC</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -2772,35 +2859,35 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>9551</v>
+        <v>9673</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
+          <t>CP2609090005</t>
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46288.00001157408</v>
+        <v>46274.00001157408</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>46304.99998842592</v>
+        <v>46303.99998842592</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>260930D84RADEG</t>
+          <t>261001FNX3QHKT</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
+          <t>CP2609090005</t>
         </is>
       </c>
       <c r="M61" t="n">
-        <v>9551</v>
+        <v>9673</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>2026-10-02 16:17:19</t>
+          <t>2026-10-02 17:47:09</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
@@ -2810,216 +2897,270 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>CP2609220002</t>
+          <t>CP2609090005</t>
         </is>
       </c>
       <c r="Q61" s="3" t="n">
-        <v>46288.00001157408</v>
+        <v>46274.00001157408</v>
       </c>
       <c r="R61" s="3" t="n">
-        <v>46304.99998842592</v>
+        <v>46303.99998842592</v>
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซท 9551</t>
+          <t>Dynamic ก.ย. Shp ราคา 9673</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
+          <t>MNL-002445</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>1199</v>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>DC2609220006</t>
-        </is>
-      </c>
-      <c r="D62" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="E62" s="3" t="n">
-        <v>46304.99998842592</v>
+        <v>2847</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>260930DWC0FFR9</t>
+          <t>261001FVHQUH0S</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>DC2609220006</t>
+          <t>CP2609280021 DC2609280008</t>
         </is>
       </c>
       <c r="M62" t="n">
-        <v>1199</v>
+        <v>2847</v>
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>2026-10-02 16:18:21</t>
+          <t>2026-10-02 16:32:59</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>CP</t>
-        </is>
-      </c>
-      <c r="P62" t="inlineStr">
-        <is>
-          <t>DC2609220006</t>
-        </is>
-      </c>
-      <c r="Q62" s="3" t="n">
-        <v>46288.00001157408</v>
-      </c>
-      <c r="R62" s="3" t="n">
-        <v>46304.99998842592</v>
-      </c>
-      <c r="S62" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1199</t>
+          <t>OC</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>MS2-000754</t>
+          <t>SP1-001113</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>375</v>
+        <v>1603</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46032</v>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>260929BD1UJHCV</t>
+          <t>261002HSH1MCYP</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>CP2609290069 DC2609290002</t>
+          <t>DC2609290041</t>
         </is>
       </c>
       <c r="M63" t="n">
-        <v>375</v>
+        <v>1603</v>
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>2026-10-02 16:35:35</t>
+          <t>2026-10-02 18:00:21</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>OC</t>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="Q63" s="3" t="n">
+        <v>46032</v>
+      </c>
+      <c r="R63" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 1603</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>MS2-000820</t>
+          <t>SP1-001449</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>225</v>
+        <v>2220</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>DC2610010003</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E64" t="n">
+        <v>46336</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>260929BD1UJHCV</t>
+          <t>2610071VPKHFM4</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>CP2609290069 DC2609290002</t>
+          <t>DC2610010003</t>
         </is>
       </c>
       <c r="M64" t="n">
-        <v>225</v>
+        <v>2220</v>
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>2026-10-02 16:35:35</t>
+          <t>2026-10-08 11:50:32</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>DC2610010003</t>
+        </is>
+      </c>
+      <c r="Q64" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R64" s="3" t="n">
+        <v>46336</v>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>Shp+Lzd+Tiktok ราคา 2220</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>MS2-000942</t>
+          <t>SP2-001778+SP2-001779</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>450</v>
+        <v>851</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>46296.0000115741</v>
+      </c>
+      <c r="E65" t="n">
+        <v>46326.9999884259</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>260929BD1UJHCV</t>
+          <t>26100839JAVCJ8</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>CP2609290069 DC2609290002</t>
+          <t>DC2609290041</t>
         </is>
       </c>
       <c r="M65" t="n">
-        <v>450</v>
+        <v>851</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>2026-10-02 16:35:35</t>
+          <t>2026-10-08 11:26:00</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="Q65" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="R65" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 851</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>SP1-001420+SP1-001421+SP1-001422+SP1-001423</t>
+          <t>SP2-001607+SP2-001754</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>9673</v>
+        <v>810</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>CP2609090005</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="n">
-        <v>46274.00001157408</v>
-      </c>
-      <c r="E66" s="3" t="n">
-        <v>46303.99998842592</v>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>46296.0000115741</v>
+      </c>
+      <c r="E66" t="n">
+        <v>46326.9999884259</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>261001FNX3QHKT</t>
+          <t>2610072GWE2YKY</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>CP2609090005</t>
+          <t>DC2609290041</t>
         </is>
       </c>
       <c r="M66" t="n">
-        <v>9673</v>
+        <v>810</v>
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>2026-10-02 17:47:09</t>
+          <t>2026-10-08 11:19:24</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
@@ -3029,319 +3170,583 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>CP2609090005</t>
+          <t>DC2609290041</t>
         </is>
       </c>
       <c r="Q66" s="3" t="n">
-        <v>46274.00001157408</v>
+        <v>46296.00001157408</v>
       </c>
       <c r="R66" s="3" t="n">
-        <v>46303.99998842592</v>
+        <v>46326.99998842592</v>
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>Dynamic ก.ย. Shp ราคา 9673</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 810</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>MNL-002445</t>
+          <t>MS2-000818</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>2847</v>
+        <v>225</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>261001FVHQUH0S</t>
+          <t>261007288HJTKT</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>CP2609280021 DC2609280008</t>
+          <t>CP2609290069 DC2609290002</t>
         </is>
       </c>
       <c r="M67" t="n">
-        <v>2847</v>
+        <v>225</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>2026-10-02 16:32:59</t>
+          <t>2026-10-08 11:12:30</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>OC</t>
+          <t>CP</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>SP1-001113</t>
+          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>1603</v>
+        <v>1052</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>DC2609290041</t>
-        </is>
-      </c>
-      <c r="D68" s="3" t="n">
-        <v>46032</v>
-      </c>
-      <c r="E68" s="3" t="n">
-        <v>46326</v>
-      </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>261002HSH1MCYP</t>
-        </is>
-      </c>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>DC2609290041</t>
-        </is>
-      </c>
-      <c r="M68" t="n">
-        <v>1603</v>
+          <t>CP2610060010</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>07/10/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>20/10/2026 23:59:59</t>
+        </is>
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>2026-10-02 18:00:21</t>
-        </is>
-      </c>
-      <c r="O68" t="inlineStr">
-        <is>
-          <t>CP</t>
+          <t>2026-10-08 11:16:15</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>DC2609290041</t>
-        </is>
-      </c>
-      <c r="Q68" s="3" t="n">
-        <v>46032</v>
-      </c>
-      <c r="R68" s="3" t="n">
-        <v>46326</v>
+          <t>CP2610060010</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>07/10/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>20/10/2026 23:59:59</t>
+        </is>
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคา 1603</t>
+          <t>FS Shp ราคาเซ็ทละ 1052</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SP1-001449</t>
+          <t>SP2-001803+SP2-001804+SP2-001805+SP2-001806</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>2220</v>
+        <v>2993</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>01/10/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>31/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>2610071NYB574H</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="M69" t="n">
+        <v>2993</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>2026-10-08 11:05:23</t>
+          <t>2026-10-08 11:46:06</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>DC2610010003</t>
-        </is>
-      </c>
-      <c r="Q69" s="3" t="n">
-        <v>46296</v>
-      </c>
-      <c r="R69" s="3" t="n">
-        <v>46336</v>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>01/10/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>31/10/2026 23:59:59</t>
+        </is>
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>Shp+Lzd+Tiktok ราคา 2220</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 2993</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>SP2-001778+SP2-001779</t>
+          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>851</v>
+        <v>1227</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>DC2609300024</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>01/10/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>31/10/2026 23:59:59</t>
+        </is>
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>2026-10-08 11:09:24</t>
+          <t>2026-10-08 11:21:10</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>DC2609290041</t>
-        </is>
-      </c>
-      <c r="Q70" s="3" t="n">
-        <v>46296.00001157408</v>
-      </c>
-      <c r="R70" s="3" t="n">
-        <v>46326.99998842592</v>
+          <t>DC2609300024</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>01/10/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>31/10/2026 23:59:59</t>
+        </is>
       </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 851</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1227</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SP2-001607+SP2-001754</t>
+          <t>SP1-001378</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>810</v>
+        <v>3042</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>CP2610020012</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>11/11/2026</t>
+        </is>
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>2026-10-08 11:10:32</t>
+          <t>2026-10-08 11:25:03</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>DC2609290041</t>
-        </is>
-      </c>
-      <c r="Q71" s="3" t="n">
-        <v>46296.00001157408</v>
-      </c>
-      <c r="R71" s="3" t="n">
-        <v>46326.99998842592</v>
+          <t>CP2610020012</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>11/11/2026</t>
+        </is>
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 810</t>
+          <t>Dynamic ต.ค. Shp ราคา 3042</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>MS2-000818</t>
+          <t>SP2-001799+SP2-001800+SP2-001801+SP2-001802</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>225</v>
-      </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>261007288HJTKT</t>
-        </is>
-      </c>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t>CP2609290069 DC2609290002</t>
-        </is>
-      </c>
-      <c r="M72" t="n">
-        <v>225</v>
+        <v>1849</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>CP2609210010</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>21/09/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>08/10/2026 23:59:59</t>
+        </is>
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>2026-10-08 11:12:30</t>
-        </is>
-      </c>
-      <c r="O72" t="inlineStr">
-        <is>
-          <t>CP</t>
+          <t>2026-10-08 11:37:15</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>CP2609210010</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>21/09/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>08/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>Dynamic ก.ย. Shp ราคาเซท 1849</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>SP2-001753+SP2-001755</t>
+          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>993</v>
+        <v>952</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>CP2610050027</t>
-        </is>
-      </c>
-      <c r="D73" s="3" t="n">
-        <v>46152.00001157408</v>
-      </c>
-      <c r="E73" s="3" t="n">
-        <v>46315.99998842592</v>
+          <t>CP2610060006</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>07/10/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>20/10/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>26100718VN19D3</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>CP2610060006</t>
+        </is>
+      </c>
+      <c r="M73" t="n">
+        <v>952</v>
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>2026-10-08 11:13:20</t>
+          <t>2026-10-08 11:40:06</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>CP2610050027</t>
-        </is>
-      </c>
-      <c r="Q73" s="3" t="n">
-        <v>46152.00001157408</v>
-      </c>
-      <c r="R73" s="3" t="n">
-        <v>46315.99998842592</v>
+          <t>CP2610060006</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>07/10/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>20/10/2026 23:59:59</t>
+        </is>
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t>FS Shp ถูกชัวร์ ราคาเซ็ทละ 993</t>
+          <t>FS Shp ราคาเซท 952</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
+          <t>SP2-001753+SP2-001755</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>1052</v>
+        <v>993</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>CP2610050027</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>05/10/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>11/11/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>5 4</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>261003K6J8B8H5</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>CP2609140012</t>
+        </is>
+      </c>
+      <c r="M74" t="n">
+        <v>993</v>
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>2026-10-08 11:16:15</t>
+          <t>2026-10-08 11:49:26</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>CP + OC</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>CP2610060010</t>
+          <t>CP2610050027</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>07/10/2026 00:00:01</t>
+          <t>05/10/2026 00:00:01</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>20/10/2026 23:59:59</t>
+          <t>11/11/2026 23:59:59</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>FS Shp ราคาเซ็ทละ 1052</t>
+          <t>FS Shp ถูกชัวร์ ราคาเซ็ทละ 993</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>SP2-001753+SP2-001755</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>993</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>CP2610050027</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>05/10/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>11/11/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:49:26</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>CP2610050027</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>05/10/2026 00:00:01</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>11/11/2026 23:59:59</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>FS Shp ถูกชัวร์ ราคาเซ็ทละ 993</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>SP4-000302</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>139</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>DC2609300024</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>261005SRV913UJ</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>DC2609300024</t>
+        </is>
+      </c>
+      <c r="M76" t="n">
+        <v>139</v>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>2026-10-08 11:52:06</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>DC2609300024</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 139</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S74"/>
+  <autoFilter ref="A1:S76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(pricing): implement CP Sonic Blow dual-mode, auto topup resolve, payment filtering & dynamic conflict resolver
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/cp_data.xlsx
+++ b/projects/auto_page/autopageMKII/tables/cp_data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$S$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$S$54</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S33"/>
+  <dimension ref="A1:S54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -537,81 +537,99 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SP2-001753+SP2-001755</t>
+          <t>PR2-000471</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1056</v>
+        <v>2274</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
+          <t>CP2610020012</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46296.00001157408</v>
+        <v>46063</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>46326.99998842592</v>
+        <v>46337</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>261006TSHP0SJ6</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>CP2610020012</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>2274</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-10-08 17:16:09</t>
+          <t>2026-10-09 15:47:26</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
+          <t>CP2610020012</t>
         </is>
       </c>
       <c r="Q2" s="3" t="n">
-        <v>46296.00001157408</v>
+        <v>46063</v>
       </c>
       <c r="R2" s="3" t="n">
-        <v>46326.99998842592</v>
+        <v>46337</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1056</t>
+          <t>Dynamic ต.ค. Shp ราคา 2274</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SP4-000302</t>
+          <t>PR3-000099</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>139</v>
+        <v>10238</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CP2609040005</t>
+          <t>CP2610070014</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46296</v>
+        <v>46304</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>46326</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>261007247UHVK3</t>
+          <t>2610095VAKA4EC</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>CP2609040005</t>
+          <t>CP2610070014</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>139</v>
+        <v>10238</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-10-08 17:52:16</t>
+          <t>2026-10-09 15:32:16</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -621,33 +639,33 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>CP2609040005</t>
+          <t>CP2610070014</t>
         </is>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>46269</v>
+        <v>46304</v>
       </c>
       <c r="R3" s="3" t="n">
-        <v>46303</v>
+        <v>46326</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Shp Fs ถูกชัวร์ ราคา139</t>
+          <t>Shp/TT เดือน ต.ค. ราคา 10238</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SP4-000302</t>
+          <t>PR5-000503</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>139</v>
+        <v>2128</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DC2609300024</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
@@ -656,14 +674,32 @@
       <c r="E4" s="3" t="n">
         <v>46326</v>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>261006W04KNW1R</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>2128</v>
+      </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-10-08 17:52:05</t>
+          <t>2026-10-09 16:20:47</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>DC2609300024</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="Q4" s="3" t="n">
@@ -674,79 +710,106 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคา 139</t>
+          <t>Shp/TT เดือน ต.ค. ราคา 2128</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PR3-000099</t>
+          <t>PR5-000582</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10430</v>
+        <v>2503</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>261005TDQDY6TH</t>
+          <t>2610083S15MCPJ</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>CP2609300041</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>10430</v>
+        <v>2503</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-10-08 17:16:57</t>
+          <t>2026-10-09 16:50:46</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
           <t>CP</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R5" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 2503</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
+          <t>PR5-000635</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>969</v>
+        <v>8671</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>CP2610020012</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46296.00001157408</v>
+        <v>46063</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>46326.99998842592</v>
+        <v>46337</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>261007288HJTKT</t>
+          <t>261006VFPUVVQ5</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>CP2610020012</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>969</v>
+        <v>8671</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-10-08 17:53:17</t>
+          <t>2026-10-09 16:17:20</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -756,201 +819,251 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>CP2610020012</t>
         </is>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>46296.00001157408</v>
+        <v>46063</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>46326.99998842592</v>
+        <v>46337</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 969</t>
+          <t>Dynamic ต.ค. Shp ราคา 8671</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SP4-000241</t>
+          <t>PR5-000667</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>405</v>
+        <v>7212</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DC2610010003</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>46296</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>46336</v>
+          <t>CP2609300041</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>26100725KET83K</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>CP2609300041</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>7212</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-10-08 17:19:27</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>DC2610010003</t>
-        </is>
-      </c>
-      <c r="Q7" s="3" t="n">
-        <v>46296</v>
-      </c>
-      <c r="R7" s="3" t="n">
-        <v>46336</v>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>Shp+Lzd+Tiktok ราคา 405</t>
+          <t>2026-10-09 16:38:23</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>AUTO_MATCH</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SP2-001748+SP2-001615+SP2-001616+SP2-001617</t>
+          <t>PR5-000673</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1330</v>
+        <v>8058</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DC2609290042</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46296.00001157408</v>
+        <v>46296</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>46326.99998842592</v>
+        <v>46326</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>261006VGXVPTEY</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>8058</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-10-08 17:20:12</t>
+          <t>2026-10-09 15:56:12</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>DC2609290042</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>46296.00001157408</v>
+        <v>46296</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>46326.99998842592</v>
+        <v>46326</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 1330</t>
+          <t>Shp/TT เดือน ต.ค. ราคา 8058</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SP2-001799+SP2-001800+SP2-001801+SP2-001802</t>
+          <t>PR5-000677</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1849</v>
+        <v>4530</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CP2609210010</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46286.00001157408</v>
+        <v>46296</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>46303.99998842592</v>
+        <v>46326</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2610083XE0YD4V</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>4530</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-10-08 17:20:57</t>
+          <t>2026-10-09 16:54:12</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>CP2609210010</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>46286.00001157408</v>
+        <v>46296</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>46303.99998842592</v>
+        <v>46326</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Dynamic ก.ย. Shp ราคาเซท 1849</t>
+          <t>Shp/TT เดือน ต.ค. ราคา 4530</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+          <t>PR5-000683</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>952</v>
+        <v>1755</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CP2610060006</t>
+          <t>DC2610020003</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46302.00001157408</v>
+        <v>46297</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>46315.99998842592</v>
+        <v>46337</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2610082P9HJV99</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>DC2610020003</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>1755</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-10-08 17:25:46</t>
+          <t>2026-10-09 16:45:56</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>CP2610060006</t>
+          <t>DC2610020003</t>
         </is>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>46302.00001157408</v>
+        <v>46297</v>
       </c>
       <c r="R10" s="3" t="n">
-        <v>46315.99998842592</v>
+        <v>46337</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>FS Shp ราคาเซท 952</t>
+          <t>Dynamic ต.ค. Shp ราคา 1755</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SP4-000196</t>
+          <t>PR5-000683</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>305</v>
+        <v>1669</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>DC2609300024</t>
+          <t>DC2609300021</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -959,14 +1072,32 @@
       <c r="E11" s="3" t="n">
         <v>46326</v>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2610071JD7K8N4</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>DC2609300021</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>1669</v>
+      </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-10-08 17:22:44</t>
+          <t>2026-10-09 16:30:18</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>DC2609300024</t>
+          <t>DC2609300021</t>
         </is>
       </c>
       <c r="Q11" s="3" t="n">
@@ -977,88 +1108,84 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคา 305</t>
+          <t>Shp/TT เดือน ต.ค. ราคา 1669</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
+          <t>PR5-000686</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1477</v>
+        <v>4983</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>46296.00001157408</v>
-      </c>
-      <c r="E12" s="3" t="n">
-        <v>46326.99998842592</v>
+          <t>CP2609300041</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>261006V0Y0CJCQ</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>CP2609300041</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>4983</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-10-08 17:23:30</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>CP2609300040</t>
-        </is>
-      </c>
-      <c r="Q12" s="3" t="n">
-        <v>46296.00001157408</v>
-      </c>
-      <c r="R12" s="3" t="n">
-        <v>46326.99998842592</v>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1477</t>
+          <t>2026-10-09 15:52:00</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SP2-001753+SP2-001755</t>
+          <t>PR6-000223</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>993</v>
+        <v>4537</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CP2610050027</t>
+          <t>CP2610020012</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46300.00001157408</v>
+        <v>46063</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>46337.99998842592</v>
+        <v>46337</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2610071U7NJ4MH</t>
+          <t>261006UJQVTNTJ</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>CP2610050027</t>
+          <t>CP2610020012</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>993</v>
+        <v>4537</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-10-08 17:46:50</t>
+          <t>2026-10-09 16:14:45</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1068,57 +1195,57 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>CP2610050027</t>
+          <t>CP2610020012</t>
         </is>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>46300.00001157408</v>
+        <v>46063</v>
       </c>
       <c r="R13" s="3" t="n">
-        <v>46337.99998842592</v>
+        <v>46337</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>FS Shp ถูกชัวร์ ราคาเซ็ทละ 993</t>
+          <t>Dynamic ต.ค. Shp ราคา 4537</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SP2-001610+SP2-001611+SP2-001612+SP2-001613</t>
+          <t>SP1-001113</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1280</v>
+        <v>1603</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
+          <t>DC2609290041</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46296.00001157408</v>
+        <v>46296</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>46326.99998842592</v>
+        <v>46326</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2610071YKH3P16</t>
+          <t>2610084KU6WNU4</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
+          <t>DC2609290041</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>1280</v>
+        <v>1603</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-10-08 17:50:28</t>
+          <t>2026-10-09 12:01:30</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1128,57 +1255,57 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
+          <t>DC2609290041</t>
         </is>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>46296.00001157408</v>
+        <v>46296</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>46326.99998842592</v>
+        <v>46326</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1280</t>
+          <t>Shp/TT เดือน ต.ค. ราคา 1603</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+          <t>SP2-001414+SP2-001415+SP2-001416+SP2-001417</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>974</v>
+        <v>1128</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>CP2610070014</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46296.00001157408</v>
+        <v>46304.00001157408</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>46326.99998842592</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>26100729ENA013</t>
+          <t>26100963TRWGR3</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>CP2610070014</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>974</v>
+        <v>1128</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-10-08 17:55:09</t>
+          <t>2026-10-09 15:41:03</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1188,197 +1315,367 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>CP2610070014</t>
         </is>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>46296.00001157408</v>
+        <v>46304.00001157408</v>
       </c>
       <c r="R15" s="3" t="n">
         <v>46326.99998842592</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 974</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1128</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SP4-000076</t>
+          <t>SP2-001610+SP2-001611+SP2-001612+SP2-001613</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>590</v>
+        <v>1280</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>46326.99998842592</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2610071JEP9U3J</t>
+          <t>26100845P38NYB</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>590</v>
+        <v>1280</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-10-08 17:36:01</t>
+          <t>2026-10-09 11:50:22</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>OC</t>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="Q16" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="R16" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1280</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SP2-001869+SP2-001870</t>
+          <t>SP2-001610+SP2-001611+SP2-001612+SP2-001613</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>921</v>
+        <v>1253</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CP2610070011</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>46304.00001157408</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>26100956M2WE0Q</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>CP2610070011</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>1253</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-10-08 17:47:27</t>
+          <t>2026-10-09 12:07:21</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>DC2609290041</t>
+          <t>CP2610070011</t>
         </is>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>46296.00001157408</v>
+        <v>46304.00001157408</v>
       </c>
       <c r="R17" s="3" t="n">
         <v>46326.99998842592</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 921</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1253</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SP1-001449</t>
+          <t>SP2-001678+SP2-001679+SP2-001680+SP2-001681</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2220</v>
+        <v>2974</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>261008513P2D80</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>2974</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-10-08 17:47:58</t>
+          <t>2026-10-09 12:06:25</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>DC2610010003</t>
+          <t>CP2609290081</t>
         </is>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>46296</v>
+        <v>46296.00001157408</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>46336</v>
+        <v>46326.99998842592</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>Shp+Lzd+Tiktok ราคา 2220</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 2974</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MS2-000818</t>
+          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>225</v>
+        <v>952</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CP2609290069 DC2609290002</t>
-        </is>
+          <t>CP2610060006</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>46302.00001157408</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>46315.99998842592</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>261007288HJTKT</t>
+          <t>26100718VN19D3</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>CP2609290069 DC2609290002</t>
+          <t>CP2610060006</t>
         </is>
       </c>
       <c r="M19" t="n">
-        <v>225</v>
+        <v>952</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-10-08 17:53:17</t>
+          <t>2026-10-09 11:43:38</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
           <t>CP</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>CP2610060006</t>
+        </is>
+      </c>
+      <c r="Q19" s="3" t="n">
+        <v>46302.00001157408</v>
+      </c>
+      <c r="R19" s="3" t="n">
+        <v>46315.99998842592</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>FS Shp ราคาเซท 952</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
+          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1052</v>
+        <v>974</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2610084C4VS82X</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>974</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-10-08 17:54:11</t>
+          <t>2026-10-09 11:58:42</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>CP2610060010</t>
+          <t>CP2609290081</t>
         </is>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>46302.00001157408</v>
+        <v>46296.00001157408</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>46315.99998842592</v>
+        <v>46326.99998842592</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>FS Shp ราคาเซ็ทละ 1052</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 974</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SP2-001753+SP2-001755</t>
+          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1056</v>
+        <v>1227</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>DC2609300024</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>261008494XV9ND</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>DC2609300024</t>
+        </is>
+      </c>
+      <c r="M21" t="n">
+        <v>1227</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-10-08 17:16:09</t>
+          <t>2026-10-09 11:54:31</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
+          <t>DC2609300024</t>
         </is>
       </c>
       <c r="Q21" s="3" t="n">
@@ -1389,269 +1686,458 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1056</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1227</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PR3-000099</t>
+          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>10430</v>
+        <v>1052</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CP2609300041</t>
-        </is>
+          <t>CP2610060010</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>46302.00001157408</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>46315.99998842592</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>261005TDQDY6TH</t>
+          <t>2610084TS30HKC</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>CP2609300041</t>
+          <t>CP2610060010</t>
         </is>
       </c>
       <c r="M22" t="n">
-        <v>10430</v>
+        <v>1052</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-10-08 17:16:57</t>
+          <t>2026-10-09 12:04:55</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
           <t>CP</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>CP2610060010</t>
+        </is>
+      </c>
+      <c r="Q22" s="3" t="n">
+        <v>46302.00001157408</v>
+      </c>
+      <c r="R22" s="3" t="n">
+        <v>46315.99998842592</v>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>FS Shp ราคาเซ็ทละ 1052</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
+          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>969</v>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>261007288HJTKT</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>CP2609290081</t>
-        </is>
-      </c>
-      <c r="M23" t="n">
-        <v>969</v>
+        <v>1199</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>DC2609220006</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>46288.00001157408</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>46304.99998842592</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-10-08 17:53:17</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>CP</t>
+          <t>2026-10-09 12:12:08</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>CP2609290081</t>
+          <t>DC2609220006</t>
         </is>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>46296.00001157408</v>
+        <v>46288.00001157408</v>
       </c>
       <c r="R23" s="3" t="n">
-        <v>46326.99998842592</v>
+        <v>46304.99998842592</v>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 969</t>
+          <t>Shp/TT เดือน ก.ย. ราคาเซ็ทละ 1199</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SP4-000241</t>
+          <t>SP2-001713+SP2-001714+SP2-001715+SP2-001716</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>405</v>
+        <v>1199</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>DC2610070012</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>46304.00001157408</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>26100956TPKHNE</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>DC2610070012</t>
+        </is>
+      </c>
+      <c r="M24" t="n">
+        <v>1199</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-10-08 17:19:27</t>
+          <t>2026-10-09 12:12:20</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>DC2610010003</t>
+          <t>DC2610070012</t>
         </is>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>46032</v>
+        <v>46304.00001157408</v>
       </c>
       <c r="R24" s="3" t="n">
-        <v>46336</v>
+        <v>46326.99998842592</v>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Shp+Lzd+Tiktok ราคา 405</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1199</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SP2-001748+SP2-001615+SP2-001616+SP2-001617</t>
+          <t>SP2-001717</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1330</v>
+        <v>425</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>DC2610010003</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>2610084EQCG957</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>DC2610010003</t>
+        </is>
+      </c>
+      <c r="M25" t="n">
+        <v>425</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-10-08 17:20:12</t>
+          <t>2026-10-09 12:00:48</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>DC2609290042</t>
+          <t>DC2610010003</t>
         </is>
       </c>
       <c r="Q25" s="3" t="n">
-        <v>46296.00001157408</v>
+        <v>46296</v>
       </c>
       <c r="R25" s="3" t="n">
-        <v>46326.99998842592</v>
+        <v>46306</v>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 1330</t>
+          <t>Shp+Lzd+Tiktok ราคา 425</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SP2-001799+SP2-001800+SP2-001801+SP2-001802</t>
+          <t>SP2-001753+SP2-001755</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1849</v>
+        <v>1056</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>2610084BHD35QS</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="M26" t="n">
+        <v>1056</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-10-08 17:20:57</t>
+          <t>2026-10-09 11:56:02</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>CP2609210010</t>
+          <t>CP2609300040</t>
         </is>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>46286.00001157408</v>
+        <v>46296.00001157408</v>
       </c>
       <c r="R26" s="3" t="n">
-        <v>46303.99998842592</v>
+        <v>46326.99998842592</v>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Dynamic ก.ย. Shp ราคาเซท 1849</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1056</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+          <t>SP2-001753+SP2-001755</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>952</v>
+        <v>993</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>CP2610050027</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>46300.00001157408</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>46337.99998842592</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>2610071CNVJU2Q</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>CP2610050027</t>
+        </is>
+      </c>
+      <c r="M27" t="n">
+        <v>993</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-10-08 17:25:46</t>
+          <t>2026-10-09 11:46:05</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>CP2610060006</t>
+          <t>CP2610050027</t>
         </is>
       </c>
       <c r="Q27" s="3" t="n">
-        <v>46302.00001157408</v>
+        <v>46300.00001157408</v>
       </c>
       <c r="R27" s="3" t="n">
-        <v>46315.99998842592</v>
+        <v>46337.99998842592</v>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>FS Shp ราคาเซท 952</t>
+          <t>FS Shp ถูกชัวร์ ราคาเซ็ทละ 993</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SP4-000196</t>
+          <t>SP2-001753+SP2-001755</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>305</v>
+        <v>1034</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CP2610070011</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>46304.00001157408</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>2610095H5YJYG4</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>CP2610070011</t>
+        </is>
+      </c>
+      <c r="M28" t="n">
+        <v>1034</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-10-08 17:22:44</t>
+          <t>2026-10-09 12:08:09</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>DC2609300024</t>
+          <t>CP2610070011</t>
         </is>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>46296</v>
+        <v>46304.00001157408</v>
       </c>
       <c r="R28" s="3" t="n">
-        <v>46326</v>
+        <v>46326.99998842592</v>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคา 305</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1034</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
+          <t>SP2-001778+SP2-001779</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1477</v>
+        <v>851</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>2610084S0WAP2B</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>DC2609290041</t>
+        </is>
+      </c>
+      <c r="M29" t="n">
+        <v>851</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-10-08 17:23:30</t>
+          <t>2026-10-09 12:04:03</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>CP</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>CP2609300040</t>
+          <t>DC2609290041</t>
         </is>
       </c>
       <c r="Q29" s="3" t="n">
@@ -1662,22 +2148,33 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1477</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 851</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SP2-001610+SP2-001611+SP2-001612+SP2-001613</t>
+          <t>SP2-001792+SP2-001793+SP2-001794+SP2-001795</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1280</v>
+        <v>1477</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>46326.99998842592</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>2610071YKH3P16</t>
+          <t>2610084EQCG957</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -1686,11 +2183,11 @@
         </is>
       </c>
       <c r="M30" t="n">
-        <v>1280</v>
+        <v>1477</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-10-08 17:50:28</t>
+          <t>2026-10-09 12:00:48</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -1711,35 +2208,46 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1280</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซ็ทละ 1477</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SP2-001753+SP2-001755</t>
+          <t>SP2-001799+SP2-001800+SP2-001801+SP2-001802</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>993</v>
+        <v>1889</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>46326.99998842592</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2610071U7NJ4MH</t>
+          <t>261008513P2D80</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>CP2610050027</t>
+          <t>CP2609290081</t>
         </is>
       </c>
       <c r="M31" t="n">
-        <v>993</v>
+        <v>1889</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-10-08 17:46:50</t>
+          <t>2026-10-09 12:06:25</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -1749,33 +2257,44 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>CP2610050027</t>
+          <t>CP2609290081</t>
         </is>
       </c>
       <c r="Q31" s="3" t="n">
-        <v>46152.00001157408</v>
+        <v>46296.00001157408</v>
       </c>
       <c r="R31" s="3" t="n">
-        <v>46337.99998842592</v>
+        <v>46326.99998842592</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>FS Shp ถูกชัวร์ ราคาเซ็ทละ 993</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 1889</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+          <t>SP2-001845+SP2-001846+SP2-001847+SP2-001848</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>974</v>
+        <v>969</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>46326.99998842592</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>26100729ENA013</t>
+          <t>2610084AXQ548E</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -1784,11 +2303,11 @@
         </is>
       </c>
       <c r="M32" t="n">
-        <v>974</v>
+        <v>969</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-10-08 17:55:09</t>
+          <t>2026-10-09 11:55:21</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -1809,35 +2328,46 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>Shp/TT เดือน ต.ค. ราคาเซท 974</t>
+          <t>Shp/TT เดือน ต.ค. ราคาเซท 969</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>MS2-000818</t>
+          <t>SP4-000196</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>225</v>
+        <v>305</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>DC2609300024</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>46326</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>261007288HJTKT</t>
+          <t>26100717549GJX</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>CP2609290069 DC2609290002</t>
+          <t>DC2609300024</t>
         </is>
       </c>
       <c r="M33" t="n">
-        <v>225</v>
+        <v>305</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-10-08 17:53:17</t>
+          <t>2026-10-09 11:41:05</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -1845,9 +2375,1262 @@
           <t>CP</t>
         </is>
       </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>DC2609300024</t>
+        </is>
+      </c>
+      <c r="Q33" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R33" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 305</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SP4-000241</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>405</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>DC2610010003</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>2610084DVJ6W6W</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>DC2610010003</t>
+        </is>
+      </c>
+      <c r="M34" t="n">
+        <v>405</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>2026-10-09 11:59:14</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>DC2610010003</t>
+        </is>
+      </c>
+      <c r="Q34" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R34" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Shp+Lzd+Tiktok ราคา 405</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SP4-000302</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>139</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>DC2609300024</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>2610084NP759P9</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>DC2609300024</t>
+        </is>
+      </c>
+      <c r="M35" t="n">
+        <v>139</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>2026-10-09 12:03:21</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>DC2609300024</t>
+        </is>
+      </c>
+      <c r="Q35" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R35" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 139</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SP4-000302</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>142</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>DC2610070012</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>2610095VAKA4EC</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>DC2610070012</t>
+        </is>
+      </c>
+      <c r="M36" t="n">
+        <v>142</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>2026-10-09 15:32:16</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>DC2610070012</t>
+        </is>
+      </c>
+      <c r="Q36" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="R36" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 142</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>PR5-000635</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>8618</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:18:47</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="Q37" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R37" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 8618</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PR6-000277</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>5304</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>261006VR7E6YBP</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="M38" t="n">
+        <v>5304</v>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:32:38</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="Q38" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R38" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 5304</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>PR6-000223</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>4410</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>2610083V0VVBCD</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="M39" t="n">
+        <v>4410</v>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:55:16</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="Q39" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R39" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 4410</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>PR5-000631</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1669</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>DC2609300021</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>2610083WPS4THV</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>DC2609300021</t>
+        </is>
+      </c>
+      <c r="M40" t="n">
+        <v>1669</v>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:55:52</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>DC2609300021</t>
+        </is>
+      </c>
+      <c r="Q40" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R40" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 1669</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>PR6-000170</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>6306</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>2610071832RHFY</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="M41" t="n">
+        <v>6306</v>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:34:39</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="Q41" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R41" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 6306</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>PR6-000279</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>6055</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>2610071BYJ7X5E</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="M42" t="n">
+        <v>6055</v>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:38:31</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="Q42" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R42" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 6055</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>PR5-000645</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>3997</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>CP2610060009</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>2610071AA2DK93</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>CP2610060009</t>
+        </is>
+      </c>
+      <c r="M43" t="n">
+        <v>3997</v>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:36:32</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>CP2610060009</t>
+        </is>
+      </c>
+      <c r="Q43" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="R43" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>FS Shp ราคา 3997</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>PR1-000584</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1252</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>DC2609300021</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>2610083PXSTGXP</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>DC2609300021</t>
+        </is>
+      </c>
+      <c r="M44" t="n">
+        <v>1252</v>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:54:34</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>DC2609300021</t>
+        </is>
+      </c>
+      <c r="Q44" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R44" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 1252</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>PR2-000471</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2165</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>2610071H7M1J0B</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="M45" t="n">
+        <v>2165</v>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:41:28</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="Q45" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R45" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 2165</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>PR5-000681</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2659</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>DC2610020005</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>46063</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>46337</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>2610071KCY80UD</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>DC2610020005</t>
+        </is>
+      </c>
+      <c r="M46" t="n">
+        <v>2659</v>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:42:05</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>DC2610020005</t>
+        </is>
+      </c>
+      <c r="Q46" s="3" t="n">
+        <v>46063</v>
+      </c>
+      <c r="R46" s="3" t="n">
+        <v>46337</v>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Dynamic ต.ค. Shp ราคา 2659</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>PR6-000446</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>6270</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CP2609290084</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>26100721GYMAWW</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>CP2609290084</t>
+        </is>
+      </c>
+      <c r="M47" t="n">
+        <v>6270</v>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:45:42</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>CP2609290084</t>
+        </is>
+      </c>
+      <c r="Q47" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R47" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 6270</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>PR5-000659</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>4625</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E48" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>26100729Q35MAX</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="M48" t="n">
+        <v>4625</v>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:48:46</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="Q48" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R48" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 4625</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>PR6-000445</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>5507</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>CP2609290084</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E49" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>261007252AEWRW</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>CP2609290084</t>
+        </is>
+      </c>
+      <c r="M49" t="n">
+        <v>5507</v>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:46:57</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>CP2609290084</t>
+        </is>
+      </c>
+      <c r="Q49" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R49" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 5507</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>PR6-000432</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>15615</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E50" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>2610083XRBVTMU</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="M50" t="n">
+        <v>15615</v>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:56:35</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>CP2609290081</t>
+        </is>
+      </c>
+      <c r="Q50" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R50" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 15615</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>PR5-000667</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>6383</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>CP2610060010</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>2610082JXTGRUJ</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>CP2610060010</t>
+        </is>
+      </c>
+      <c r="M51" t="n">
+        <v>6383</v>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:50:36</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>CP2610060010</t>
+        </is>
+      </c>
+      <c r="Q51" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="R51" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>FS Shp ราคา 6383</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>PR2-000495</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>4565</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>2610082K71NDWN</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="M52" t="n">
+        <v>4565</v>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:51:13</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="Q52" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R52" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 4565</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>PR5-000627</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>3183</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>2610083MKMP7HY</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="M53" t="n">
+        <v>3183</v>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>2026-10-09 17:53:52</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>CP2609300040</t>
+        </is>
+      </c>
+      <c r="Q53" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R53" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Shp/TT เดือน ต.ค. ราคา 3183</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>PR3-000099</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>10430</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>CP2609300041</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>2610083WD60HJX</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>CP2609300041</t>
+        </is>
+      </c>
+      <c r="M54" t="n">
+        <v>10430</v>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:52:49</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>AUTO_MATCH</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>CP2610070014</t>
+        </is>
+      </c>
+      <c r="Q54" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="R54" s="3" t="n">
+        <v>46326</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S33"/>
+  <autoFilter ref="A1:S54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(accel & pricing): record manual invoices to Processed_Logs with accel_file, add seller voucher detail & combo coupon resolve
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/cp_data.xlsx
+++ b/projects/auto_page/autopageMKII/tables/cp_data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$S$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$S$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S54"/>
+  <dimension ref="A1:S81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3629,8 +3629,1164 @@
         <v>46326</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>MNL-002120</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>7225</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CP2609300027</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>261003K7HY2GGE</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>CP2609300027</t>
+        </is>
+      </c>
+      <c r="M55" t="n">
+        <v>7225</v>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>2026-10-10 13:42:45</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>AUTO_MATCH</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>CP2609300027</t>
+        </is>
+      </c>
+      <c r="Q55" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R55" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>promotion xmn viewsonic period 1-31 oct 2026  topup all store (viewsonic sup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>MNL-002445</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>2847</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>CP2609280021 DC2609280008</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>46308.99998842592</v>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>261006UWKM892H</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>CP2609280021 DC2609280008</t>
+        </is>
+      </c>
+      <c r="M56" t="n">
+        <v>2847</v>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>2026-10-10 13:07:55</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>AUTO_MATCH</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>CP2609280021 DC2609280008</t>
+        </is>
+      </c>
+      <c r="Q56" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="R56" s="3" t="n">
+        <v>46308.99998842592</v>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>Promotion xdt acer period 1-13 Oct 26 Topup All Store  BG250053, promotion xdt xmn period 01-31 oct 2026 topup all store dc months all brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>MNL-002423</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>15857</v>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>2026-10-10 12:26:27</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>ไม่มี pattern, cp/dcที่พบ: 2 อัน</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>MNL-002416</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>2829</v>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>2026-10-10 12:27:05</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>ไม่มี pattern, cp/dcที่พบ: 1 อัน</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>MNL-002550</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>2977</v>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>2026-10-10 12:27:38</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>ไม่มี pattern, cp/dcที่พบ: 2 อัน</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>MNL-002358</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>2157</v>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>2026-10-10 12:29:03</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>CP2609290086 CP2610090037</t>
+        </is>
+      </c>
+      <c r="Q60" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R60" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>ใช้คูปอง dynamic นี้ราคาขายยิงขึ้น 2157</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>MNL-002403</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>6372</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="M61" t="n">
+        <v>6505</v>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>2026-10-10 17:22:50</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>AUTO_MATCH</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="Q61" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R61" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>promotion xdt xmn period 01-31 oct 2026 topup all store dc months all brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>MNL-002420</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>3724</v>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:46:54</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="Q62" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R62" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>promotion xdt xmn period 01-31 oct 2026 topup all store dc months all brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>MNL-002404</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>6792</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>26100714TQ0CEY</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="M63" t="n">
+        <v>6792</v>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>2026-10-10 10:22:39</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>OC</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>MNL-002507</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>2187</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>CP2610100002</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>2026-10-10 10:23:11</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>CP2610100002</t>
+        </is>
+      </c>
+      <c r="Q64" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R64" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>ใช้คูปอง dynamic นี้ราคาขายยิงขึ้น 2187</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>MNL-002584</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>2610071822BPS6</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="M65" t="n">
+        <v>2023</v>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>2026-10-10 11:41:31</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>AUTO_MATCH</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="Q65" s="3" t="n">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>MNL-002489</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>2869</v>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>2026-10-10 10:24:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>MNL-002505</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>7461</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>2610071AX38J9S</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="M67" t="n">
+        <v>7461</v>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:51:06</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>AUTO_MATCH</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="Q67" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R67" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>promotion xdt xmn period 01-31 oct 2026 topup all store dc months all brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>MNL-002555</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>3460</v>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>2026-10-10 10:25:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>MNL-002478</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>3133</v>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>2026-10-10 10:25:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>MNL-002483</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>3405</v>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>2026-10-10 10:26:27</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>CP2610050031</t>
+        </is>
+      </c>
+      <c r="Q70" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="R70" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>promotion xmn lg period 05-11 oct 26 addon online (bg260024)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>MNL-002409</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>2922</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>2610107P8TY5NB</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="M71" t="n">
+        <v>2922</v>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>2026-10-10 17:51:29</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="Q71" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R71" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>promotion xdt xmn period 01-31 oct 2026 topup all store dc months all brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>MNL-002420</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>3601</v>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>2026-10-10 17:31:59</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>ไม่มี pattern, cp/dcที่พบ: 2 อัน</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>MNL-002511</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>3691</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>CP2609290086 DC2609280008</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E73" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>2610107P9GX020</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>CP2609290086 DC2609280008</t>
+        </is>
+      </c>
+      <c r="M73" t="n">
+        <v>3691</v>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:47:45</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>AUTO_MATCH</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>CP2609290086 DC2609280008</t>
+        </is>
+      </c>
+      <c r="Q73" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="R73" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>promotion xdt xmn lenovo period 1-30 oct 2026 topup all store bg260044, promotion xdt xmn period 01-31 oct 2026 topup all store dc months all brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>MNL-002498</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>3548</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>CP2609280028 DC2609280008</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="E74" s="3" t="n">
+        <v>46308.99998842592</v>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>2610107P9E19NE</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>CP2609280028 DC2609280008</t>
+        </is>
+      </c>
+      <c r="M74" t="n">
+        <v>3548</v>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:48:44</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>OC</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>CP2609280028 DC2609280008</t>
+        </is>
+      </c>
+      <c r="Q74" s="3" t="n">
+        <v>46296.00001157408</v>
+      </c>
+      <c r="R74" s="3" t="n">
+        <v>46308.99998842592</v>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>Promotion xmn acer  period 1-13 Oct 26 topup all store  IABP260665, promotion xdt xmn period 01-31 oct 2026 topup all store dc months all brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>MNL-002483</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>3476</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E75" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>2610107PFGN2MY</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="M75" t="n">
+        <v>3476</v>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:49:23</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>AUTO_MATCH</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="Q75" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R75" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>promotion xdt xmn period 01-31 oct 2026 topup all store dc months all brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>MNL-002484</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>4648</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>CP2610060002</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46301.00001157408</v>
+      </c>
+      <c r="E76" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>26100979W27913</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>CP2610060002</t>
+        </is>
+      </c>
+      <c r="M76" t="n">
+        <v>4648</v>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:50:22</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>OC</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>CP2610060002</t>
+        </is>
+      </c>
+      <c r="Q76" s="3" t="n">
+        <v>46301.00001157408</v>
+      </c>
+      <c r="R76" s="3" t="n">
+        <v>46326.99998842592</v>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>Promotion xmn lg period 06-31 oct 2026 topup all store bg250024</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>MNL-002505</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>7617</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E77" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>2610096GCN7NY6</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="M77" t="n">
+        <v>7617</v>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:51:26</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>OC</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="Q77" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R77" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>promotion xdt xmn period 01-31 oct 2026 topup all store dc months all brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>MNL-002403</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>6505</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E78" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>2610107P9A8HRX</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="M78" t="n">
+        <v>6505</v>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>2026-10-10 17:22:46</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>AUTO_MATCH</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="Q78" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R78" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>promotion xdt xmn period 01-31 oct 2026 topup all store dc months all brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>MNL-002371</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>8351</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E79" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>2610096EP9QSXE</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="M79" t="n">
+        <v>8351</v>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>2026-10-10 17:22:48</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>AUTO_MATCH</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>DC2609280008</t>
+        </is>
+      </c>
+      <c r="Q79" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="R79" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>promotion xdt xmn period 01-31 oct 2026 topup all store dc months all brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>MNL-002437</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>5619</v>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>2026-10-10 16:54:17</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>ไม่มี pattern, cp/dcที่พบ: 2 อัน</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>MNL-002409</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>2863</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>CP2610100002 DC2609280008</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>2610107PUSHD2B</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>CP2610100002 DC2609280008</t>
+        </is>
+      </c>
+      <c r="M81" t="n">
+        <v>2863</v>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>2026-10-10 17:52:49</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>CP2610100002 DC2609280008</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>ใช้คูปอง dynamic นี้ราคาขายยิงขึ้น 2187, promotion xdt xmn period 01-31 oct 2026 topup all store dc months all brand</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S54"/>
+  <autoFilter ref="A1:S81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>